<commit_message>
Update binary files and enhance dashboard functionality
- Updated multiple binary files including `ErectionCompiled_Output.xlsx`, `ProdDailyExpandedSingles.parquet`, `ProjectBaselines.parquet`, `ProjectDetails.parquet`, and `StringingCompiled_Output.xlsx` to reflect recent changes in data processing.
- Deleted outdated DPR Excel files to clean up the project directory.
- Enhanced chart generation in `dashboard/charts.py` to support axis title and unit label overrides for improved data visualization.
- Improved handling of stringing metrics in `dashboard/stringing.py` to ensure accurate calculations based on selected value columns.
</commit_message>
<xml_diff>
--- a/Raw Data/Micro Plans/November 2025/Micro Plan - TA-418 Nov'25.xlsx
+++ b/Raw Data/Micro Plans/November 2025/Micro Plan - TA-418 Nov'25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\Micro Plans\November 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD672C04-A615-47EE-BAE1-B5900DFFBC61}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7DE310-4FF0-482E-8F1E-5B8361E39611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="183">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="340" uniqueCount="182">
   <si>
     <t>Project Code</t>
   </si>
@@ -582,12 +582,6 @@
     <t>41/0</t>
   </si>
   <si>
-    <t>D1</t>
-  </si>
-  <si>
-    <t>D2</t>
-  </si>
-  <si>
     <t>A</t>
   </si>
   <si>
@@ -595,6 +589,9 @@
   </si>
   <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>MANUAL</t>
   </si>
 </sst>
 </file>
@@ -1954,9 +1951,63 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1972,51 +2023,6 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2044,26 +2050,17 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="172">
@@ -2778,6 +2775,16 @@
     </dxf>
     <dxf>
       <font>
+        <color indexed="17"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="42"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color indexed="20"/>
       </font>
       <fill>
@@ -2800,16 +2807,6 @@
       <font>
         <color indexed="20"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="17"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="42"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -3631,137 +3628,137 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="177" t="s">
+      <c r="A18" s="195" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="177" t="s">
+      <c r="B18" s="195" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="174" t="s">
+      <c r="C18" s="191" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="177" t="s">
+      <c r="D18" s="195" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="174" t="s">
+      <c r="E18" s="191" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="174" t="s">
+      <c r="F18" s="191" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="177" t="s">
+      <c r="G18" s="195" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="189" t="s">
+      <c r="H18" s="182" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="189"/>
-      <c r="J18" s="189"/>
-      <c r="K18" s="189"/>
-      <c r="L18" s="189"/>
-      <c r="M18" s="189"/>
-      <c r="N18" s="189"/>
-      <c r="O18" s="189"/>
-      <c r="P18" s="182" t="s">
+      <c r="I18" s="182"/>
+      <c r="J18" s="182"/>
+      <c r="K18" s="182"/>
+      <c r="L18" s="182"/>
+      <c r="M18" s="182"/>
+      <c r="N18" s="182"/>
+      <c r="O18" s="182"/>
+      <c r="P18" s="185" t="s">
         <v>19</v>
       </c>
-      <c r="R18" s="174" t="s">
+      <c r="R18" s="191" t="s">
         <v>36</v>
       </c>
-      <c r="T18" s="183" t="s">
+      <c r="T18" s="186" t="s">
         <v>31</v>
       </c>
-      <c r="U18" s="184"/>
-      <c r="V18" s="184"/>
-      <c r="W18" s="184"/>
-      <c r="X18" s="184"/>
-      <c r="Y18" s="185"/>
-      <c r="AA18" s="183" t="s">
+      <c r="U18" s="187"/>
+      <c r="V18" s="187"/>
+      <c r="W18" s="187"/>
+      <c r="X18" s="187"/>
+      <c r="Y18" s="188"/>
+      <c r="AA18" s="186" t="s">
         <v>30</v>
       </c>
-      <c r="AB18" s="184"/>
-      <c r="AC18" s="184"/>
-      <c r="AD18" s="184"/>
-      <c r="AE18" s="184"/>
-      <c r="AF18" s="185"/>
-      <c r="AG18" s="186" t="s">
+      <c r="AB18" s="187"/>
+      <c r="AC18" s="187"/>
+      <c r="AD18" s="187"/>
+      <c r="AE18" s="187"/>
+      <c r="AF18" s="188"/>
+      <c r="AG18" s="189" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="178"/>
-      <c r="B19" s="178"/>
-      <c r="C19" s="175"/>
-      <c r="D19" s="178"/>
-      <c r="E19" s="175"/>
-      <c r="F19" s="175"/>
-      <c r="G19" s="178"/>
-      <c r="H19" s="194" t="s">
+      <c r="A19" s="196"/>
+      <c r="B19" s="196"/>
+      <c r="C19" s="193"/>
+      <c r="D19" s="196"/>
+      <c r="E19" s="193"/>
+      <c r="F19" s="193"/>
+      <c r="G19" s="196"/>
+      <c r="H19" s="181" t="s">
         <v>9</v>
       </c>
-      <c r="I19" s="194"/>
-      <c r="J19" s="194" t="s">
+      <c r="I19" s="181"/>
+      <c r="J19" s="181" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="194"/>
-      <c r="L19" s="194" t="s">
+      <c r="K19" s="181"/>
+      <c r="L19" s="181" t="s">
         <v>13</v>
       </c>
-      <c r="M19" s="194"/>
-      <c r="N19" s="190" t="s">
+      <c r="M19" s="181"/>
+      <c r="N19" s="179" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="190" t="s">
+      <c r="O19" s="179" t="s">
         <v>14</v>
       </c>
-      <c r="P19" s="182"/>
-      <c r="R19" s="188"/>
-      <c r="T19" s="180" t="s">
+      <c r="P19" s="185"/>
+      <c r="R19" s="192"/>
+      <c r="T19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="U19" s="180" t="s">
+      <c r="U19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="V19" s="180" t="s">
+      <c r="V19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="W19" s="180" t="s">
+      <c r="W19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="X19" s="180" t="s">
+      <c r="X19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="Y19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AA19" s="180" t="s">
+      <c r="AA19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="AB19" s="180" t="s">
+      <c r="AB19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="AC19" s="180" t="s">
+      <c r="AC19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="AD19" s="180" t="s">
+      <c r="AD19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="AE19" s="180" t="s">
+      <c r="AE19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="AF19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AG19" s="187"/>
+      <c r="AG19" s="190"/>
     </row>
     <row r="20" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="179"/>
-      <c r="B20" s="178"/>
-      <c r="C20" s="175"/>
-      <c r="D20" s="178"/>
-      <c r="E20" s="176"/>
-      <c r="F20" s="176"/>
-      <c r="G20" s="178"/>
+      <c r="A20" s="197"/>
+      <c r="B20" s="196"/>
+      <c r="C20" s="193"/>
+      <c r="D20" s="196"/>
+      <c r="E20" s="194"/>
+      <c r="F20" s="194"/>
+      <c r="G20" s="196"/>
       <c r="H20" s="93" t="s">
         <v>10</v>
       </c>
@@ -3780,25 +3777,25 @@
       <c r="M20" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="191"/>
-      <c r="O20" s="191"/>
+      <c r="N20" s="180"/>
+      <c r="O20" s="180"/>
       <c r="P20" s="44" t="s">
         <v>50</v>
       </c>
       <c r="R20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="T20" s="181"/>
-      <c r="U20" s="181"/>
-      <c r="V20" s="181"/>
-      <c r="W20" s="181"/>
-      <c r="X20" s="181"/>
+      <c r="T20" s="184"/>
+      <c r="U20" s="184"/>
+      <c r="V20" s="184"/>
+      <c r="W20" s="184"/>
+      <c r="X20" s="184"/>
       <c r="Y20" s="19"/>
-      <c r="AA20" s="181"/>
-      <c r="AB20" s="181"/>
-      <c r="AC20" s="181"/>
-      <c r="AD20" s="181"/>
-      <c r="AE20" s="181"/>
+      <c r="AA20" s="184"/>
+      <c r="AB20" s="184"/>
+      <c r="AC20" s="184"/>
+      <c r="AD20" s="184"/>
+      <c r="AE20" s="184"/>
       <c r="AF20" s="19" t="s">
         <v>50</v>
       </c>
@@ -4069,7 +4066,7 @@
       <c r="D25" s="85"/>
       <c r="E25" s="100"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="192"/>
+      <c r="G25" s="177"/>
       <c r="H25" s="98"/>
       <c r="I25" s="98"/>
       <c r="J25" s="98"/>
@@ -4127,7 +4124,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="101"/>
       <c r="F26" s="96"/>
-      <c r="G26" s="193"/>
+      <c r="G26" s="178"/>
       <c r="H26" s="98"/>
       <c r="I26" s="98"/>
       <c r="J26" s="98"/>
@@ -4482,16 +4479,13 @@
     <filterColumn colId="13" showButton="0"/>
   </autoFilter>
   <mergeCells count="29">
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="L19:M19"/>
-    <mergeCell ref="H18:O18"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
     <mergeCell ref="X19:X20"/>
     <mergeCell ref="P18:P19"/>
     <mergeCell ref="AA18:AF18"/>
@@ -4504,13 +4498,16 @@
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="T18:Y18"/>
     <mergeCell ref="T19:T20"/>
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="H18:O18"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="L19:M19"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B21">
@@ -4585,17 +4582,17 @@
     <cfRule type="expression" dxfId="58" priority="1243" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$123, B26)+COUNTIF($D$142:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="1244" stopIfTrue="1">
+    <cfRule type="expression" dxfId="57" priority="1245" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="1245" stopIfTrue="1">
+    <cfRule type="expression" dxfId="56" priority="1246" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="1246" stopIfTrue="1">
+    <cfRule type="expression" dxfId="55" priority="1247" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$474:$D$65380, B26)+COUNTIF($D$454:$D$455, B26)+COUNTIF($D$416:$D$417, B26)+COUNTIF($D$374:$D$377, B26)+COUNTIF($D$351:$D$352, B26)+COUNTIF($D$324:$D$325, B26)+COUNTIF($D$303:$D$303, B26)+COUNTIF($D$288:$D$289, B26)+COUNTIF($D$263:$D$263, B26)+COUNTIF($D$252:$D$253, B26)+COUNTIF($D$233:$D$234, B26)+COUNTIF($D$51:$D$218, B26)+COUNTIF($D$219:$D$220, B26)+COUNTIF($D$1:$D$50, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="54" priority="1244" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="54" priority="1247" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$474:$D$65380, B26)+COUNTIF($D$454:$D$455, B26)+COUNTIF($D$416:$D$417, B26)+COUNTIF($D$374:$D$377, B26)+COUNTIF($D$351:$D$352, B26)+COUNTIF($D$324:$D$325, B26)+COUNTIF($D$303:$D$303, B26)+COUNTIF($D$288:$D$289, B26)+COUNTIF($D$263:$D$263, B26)+COUNTIF($D$252:$D$253, B26)+COUNTIF($D$233:$D$234, B26)+COUNTIF($D$51:$D$218, B26)+COUNTIF($D$219:$D$220, B26)+COUNTIF($D$1:$D$50, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
@@ -4612,55 +4609,55 @@
     <cfRule type="duplicateValues" dxfId="47" priority="347"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4">
-    <cfRule type="expression" dxfId="46" priority="1220" stopIfTrue="1">
+    <cfRule type="expression" dxfId="46" priority="1221" stopIfTrue="1">
+      <formula>AND(COUNTIF($C$1:$C$65460, L4)+COUNTIF(#REF!, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="1220" stopIfTrue="1">
       <formula>AND(COUNTIF($C$314:$C$65460, L4)+COUNTIF($C$294:$C$295, L4)+COUNTIF($C$256:$C$257, L4)+COUNTIF($C$214:$C$217, L4)+COUNTIF($C$191:$C$192, L4)+COUNTIF($C$164:$C$165, L4)+COUNTIF($C$143:$C$143, L4)+COUNTIF($C$128:$C$129, L4)+COUNTIF($C$103:$C$103, L4)+COUNTIF($C$92:$C$93, L4)+COUNTIF($C$73:$C$74, L4)+COUNTIF($C$29:$C$56, L4)+COUNTIF($C$58:$C$60, L4)+COUNTIF($C$1:$C$27, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="45" priority="1221" stopIfTrue="1">
-      <formula>AND(COUNTIF($C$1:$C$65460, L4)+COUNTIF(#REF!, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4">
-    <cfRule type="expression" dxfId="44" priority="1222" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="43" priority="1223" stopIfTrue="1">
+    <cfRule type="expression" dxfId="44" priority="1223" stopIfTrue="1">
       <formula>AND(COUNTIF($D$314:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="1224" stopIfTrue="1">
+    <cfRule type="expression" dxfId="43" priority="1224" stopIfTrue="1">
       <formula>AND(COUNTIF($D$294:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="1225" stopIfTrue="1">
+    <cfRule type="expression" dxfId="42" priority="1225" stopIfTrue="1">
       <formula>AND(COUNTIF($D$256:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="1226" stopIfTrue="1">
+    <cfRule type="expression" dxfId="41" priority="1226" stopIfTrue="1">
       <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="1227" stopIfTrue="1">
+    <cfRule type="expression" dxfId="40" priority="1227" stopIfTrue="1">
       <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="1228" stopIfTrue="1">
+    <cfRule type="expression" dxfId="39" priority="1228" stopIfTrue="1">
       <formula>AND(COUNTIF($D$191:$D$65460, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="1229" stopIfTrue="1">
+    <cfRule type="expression" dxfId="38" priority="1229" stopIfTrue="1">
       <formula>AND(COUNTIF($F$369:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$352:$F$353, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="1230" stopIfTrue="1">
+    <cfRule type="expression" dxfId="37" priority="1230" stopIfTrue="1">
       <formula>AND(COUNTIF($F$352:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="1231" stopIfTrue="1">
+    <cfRule type="expression" dxfId="36" priority="1231" stopIfTrue="1">
       <formula>AND(COUNTIF($F$332:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="1232" stopIfTrue="1">
+    <cfRule type="expression" dxfId="35" priority="1232" stopIfTrue="1">
       <formula>AND(COUNTIF($F$294:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="1233" stopIfTrue="1">
+    <cfRule type="expression" dxfId="34" priority="1233" stopIfTrue="1">
       <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="1234" stopIfTrue="1">
+    <cfRule type="expression" dxfId="33" priority="1234" stopIfTrue="1">
       <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="31" priority="1235" stopIfTrue="1">
+    <cfRule type="expression" dxfId="32" priority="1235" stopIfTrue="1">
       <formula>AND(COUNTIF($F$229:$F$65454, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="31" priority="1222" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -4781,7 +4778,7 @@
       <c r="Q4" s="70">
         <v>0</v>
       </c>
-      <c r="R4" s="195" t="s">
+      <c r="R4" s="198" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4824,14 +4821,14 @@
       <c r="Q5" s="70">
         <v>0</v>
       </c>
-      <c r="R5" s="196"/>
+      <c r="R5" s="199"/>
     </row>
     <row r="6" spans="2:18" s="75" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="197" t="s">
+      <c r="B6" s="200" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="198"/>
-      <c r="D6" s="199"/>
+      <c r="C6" s="201"/>
+      <c r="D6" s="202"/>
       <c r="E6" s="73">
         <v>160</v>
       </c>
@@ -6329,64 +6326,64 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B1" s="200" t="s">
+      <c r="B1" s="203" t="s">
         <v>158</v>
       </c>
-      <c r="C1" s="200"/>
-      <c r="D1" s="200"/>
-      <c r="E1" s="200"/>
-      <c r="F1" s="200"/>
-      <c r="G1" s="200"/>
-      <c r="H1" s="200"/>
-      <c r="I1" s="200"/>
-      <c r="J1" s="200"/>
-      <c r="K1" s="200"/>
-      <c r="L1" s="200"/>
+      <c r="C1" s="203"/>
+      <c r="D1" s="203"/>
+      <c r="E1" s="203"/>
+      <c r="F1" s="203"/>
+      <c r="G1" s="203"/>
+      <c r="H1" s="203"/>
+      <c r="I1" s="203"/>
+      <c r="J1" s="203"/>
+      <c r="K1" s="203"/>
+      <c r="L1" s="203"/>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B2" s="201" t="s">
+      <c r="B2" s="204" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="201"/>
-      <c r="D2" s="201"/>
-      <c r="E2" s="201"/>
-      <c r="F2" s="201"/>
-      <c r="G2" s="201"/>
-      <c r="H2" s="201"/>
-      <c r="I2" s="201"/>
-      <c r="J2" s="201"/>
-      <c r="K2" s="201"/>
-      <c r="L2" s="201"/>
+      <c r="C2" s="204"/>
+      <c r="D2" s="204"/>
+      <c r="E2" s="204"/>
+      <c r="F2" s="204"/>
+      <c r="G2" s="204"/>
+      <c r="H2" s="204"/>
+      <c r="I2" s="204"/>
+      <c r="J2" s="204"/>
+      <c r="K2" s="204"/>
+      <c r="L2" s="204"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B3" s="202" t="s">
+      <c r="B3" s="205" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="202"/>
-      <c r="D3" s="202"/>
-      <c r="E3" s="202"/>
-      <c r="F3" s="202"/>
-      <c r="G3" s="202"/>
-      <c r="H3" s="202"/>
-      <c r="I3" s="202"/>
-      <c r="J3" s="202"/>
-      <c r="K3" s="202"/>
-      <c r="L3" s="202"/>
+      <c r="C3" s="205"/>
+      <c r="D3" s="205"/>
+      <c r="E3" s="205"/>
+      <c r="F3" s="205"/>
+      <c r="G3" s="205"/>
+      <c r="H3" s="205"/>
+      <c r="I3" s="205"/>
+      <c r="J3" s="205"/>
+      <c r="K3" s="205"/>
+      <c r="L3" s="205"/>
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="203" t="s">
+      <c r="B4" s="206" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="203"/>
-      <c r="D4" s="203"/>
-      <c r="E4" s="203"/>
-      <c r="F4" s="203"/>
-      <c r="G4" s="203"/>
-      <c r="H4" s="203"/>
-      <c r="I4" s="203"/>
-      <c r="J4" s="203"/>
-      <c r="K4" s="203"/>
-      <c r="L4" s="203"/>
+      <c r="C4" s="206"/>
+      <c r="D4" s="206"/>
+      <c r="E4" s="206"/>
+      <c r="F4" s="206"/>
+      <c r="G4" s="206"/>
+      <c r="H4" s="206"/>
+      <c r="I4" s="206"/>
+      <c r="J4" s="206"/>
+      <c r="K4" s="206"/>
+      <c r="L4" s="206"/>
     </row>
     <row r="5" spans="2:16" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B5" s="156" t="s">
@@ -6403,230 +6400,230 @@
       <c r="K5" s="158"/>
     </row>
     <row r="6" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B6" s="208" t="s">
+      <c r="B6" s="174" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="208" t="s">
+      <c r="C6" s="174" t="s">
         <v>163</v>
       </c>
-      <c r="D6" s="208" t="s">
+      <c r="D6" s="174" t="s">
         <v>164</v>
       </c>
-      <c r="E6" s="208" t="s">
+      <c r="E6" s="174" t="s">
         <v>165</v>
       </c>
-      <c r="F6" s="208" t="s">
+      <c r="F6" s="174" t="s">
         <v>166</v>
       </c>
-      <c r="G6" s="208" t="s">
+      <c r="G6" s="174" t="s">
         <v>167</v>
       </c>
-      <c r="H6" s="208" t="s">
+      <c r="H6" s="174" t="s">
         <v>116</v>
       </c>
-      <c r="I6" s="208" t="s">
+      <c r="I6" s="174" t="s">
         <v>117</v>
       </c>
-      <c r="J6" s="208" t="s">
+      <c r="J6" s="174" t="s">
         <v>118</v>
       </c>
-      <c r="K6" s="208" t="s">
+      <c r="K6" s="174" t="s">
         <v>168</v>
       </c>
-      <c r="L6" s="208" t="s">
+      <c r="L6" s="174" t="s">
         <v>169</v>
       </c>
-      <c r="M6" s="208" t="s">
+      <c r="M6" s="174" t="s">
         <v>108</v>
       </c>
-      <c r="N6" s="208" t="s">
+      <c r="N6" s="174" t="s">
         <v>170</v>
       </c>
-      <c r="O6" s="208" t="s">
+      <c r="O6" s="174" t="s">
         <v>105</v>
       </c>
-      <c r="P6" s="208" t="s">
+      <c r="P6" s="174" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B7" s="209">
+      <c r="B7" s="175">
         <v>1</v>
       </c>
-      <c r="C7" s="209" t="s">
+      <c r="C7" s="175" t="s">
         <v>171</v>
       </c>
-      <c r="D7" s="209" t="s">
+      <c r="D7" s="175" t="s">
         <v>172</v>
       </c>
-      <c r="E7" s="209">
+      <c r="E7" s="175">
         <v>0.48</v>
       </c>
-      <c r="F7" s="209" t="s">
+      <c r="F7" s="175" t="s">
         <v>173</v>
       </c>
-      <c r="G7" s="209">
-        <v>0</v>
-      </c>
-      <c r="H7" s="210">
+      <c r="G7" s="175">
+        <v>0</v>
+      </c>
+      <c r="H7" s="176">
         <v>45960</v>
       </c>
-      <c r="I7" s="210">
+      <c r="I7" s="176">
         <v>45962</v>
       </c>
-      <c r="J7" s="210">
+      <c r="J7" s="176">
         <v>45964</v>
       </c>
-      <c r="K7" s="210">
+      <c r="K7" s="176">
         <v>45966</v>
       </c>
-      <c r="L7" s="209" t="s">
+      <c r="L7" s="8" t="s">
+        <v>181</v>
+      </c>
+      <c r="M7" s="175" t="s">
+        <v>160</v>
+      </c>
+      <c r="N7" s="175"/>
+      <c r="O7" s="175" t="s">
         <v>178</v>
       </c>
-      <c r="M7" s="209" t="s">
+      <c r="P7" s="175" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="8" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B8" s="175">
+        <v>2</v>
+      </c>
+      <c r="C8" s="175" t="s">
+        <v>174</v>
+      </c>
+      <c r="D8" s="175" t="s">
+        <v>171</v>
+      </c>
+      <c r="E8" s="175">
+        <v>4.4800000000000004</v>
+      </c>
+      <c r="F8" s="175" t="s">
+        <v>173</v>
+      </c>
+      <c r="G8" s="175">
+        <v>11</v>
+      </c>
+      <c r="H8" s="176">
+        <v>45977</v>
+      </c>
+      <c r="I8" s="176">
+        <v>45966</v>
+      </c>
+      <c r="J8" s="176">
+        <v>45974</v>
+      </c>
+      <c r="K8" s="176">
+        <v>45976</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="M8" s="175" t="s">
         <v>160</v>
       </c>
-      <c r="N7" s="209"/>
-      <c r="O7" s="209" t="s">
+      <c r="N8" s="175"/>
+      <c r="O8" s="175" t="s">
+        <v>178</v>
+      </c>
+      <c r="P8" s="175" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="9" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B9" s="175">
+        <v>3</v>
+      </c>
+      <c r="C9" s="175" t="s">
+        <v>175</v>
+      </c>
+      <c r="D9" s="175" t="s">
+        <v>174</v>
+      </c>
+      <c r="E9" s="175">
+        <v>1.98</v>
+      </c>
+      <c r="F9" s="175" t="s">
+        <v>173</v>
+      </c>
+      <c r="G9" s="175">
+        <v>4</v>
+      </c>
+      <c r="H9" s="176">
+        <v>45984</v>
+      </c>
+      <c r="I9" s="176">
+        <v>45976</v>
+      </c>
+      <c r="J9" s="176">
+        <v>45982</v>
+      </c>
+      <c r="K9" s="176">
+        <v>45984</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="M9" s="175" t="s">
+        <v>160</v>
+      </c>
+      <c r="N9" s="175"/>
+      <c r="O9" s="175" t="s">
         <v>180</v>
       </c>
-      <c r="P7" s="209" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="8" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B8" s="209">
-        <v>2</v>
-      </c>
-      <c r="C8" s="209" t="s">
-        <v>174</v>
-      </c>
-      <c r="D8" s="209" t="s">
-        <v>171</v>
-      </c>
-      <c r="E8" s="209">
-        <v>4.4800000000000004</v>
-      </c>
-      <c r="F8" s="209" t="s">
+      <c r="P9" s="175" t="s">
+        <v>179</v>
+      </c>
+    </row>
+    <row r="10" spans="2:16" ht="29" x14ac:dyDescent="0.35">
+      <c r="B10" s="175">
+        <v>4</v>
+      </c>
+      <c r="C10" s="175" t="s">
+        <v>176</v>
+      </c>
+      <c r="D10" s="175" t="s">
+        <v>177</v>
+      </c>
+      <c r="E10" s="175">
+        <v>2.46</v>
+      </c>
+      <c r="F10" s="175" t="s">
         <v>173</v>
       </c>
-      <c r="G8" s="209">
-        <v>11</v>
-      </c>
-      <c r="H8" s="210">
-        <v>45977</v>
-      </c>
-      <c r="I8" s="210">
-        <v>45966</v>
-      </c>
-      <c r="J8" s="210">
-        <v>45974</v>
-      </c>
-      <c r="K8" s="210">
-        <v>45976</v>
-      </c>
-      <c r="L8" s="209" t="s">
-        <v>178</v>
-      </c>
-      <c r="M8" s="209" t="s">
+      <c r="G10" s="175">
+        <v>5</v>
+      </c>
+      <c r="H10" s="176">
+        <v>45971</v>
+      </c>
+      <c r="I10" s="176">
+        <v>45984</v>
+      </c>
+      <c r="J10" s="176">
+        <v>45991</v>
+      </c>
+      <c r="K10" s="176">
+        <v>45993</v>
+      </c>
+      <c r="L10" s="8" t="s">
+        <v>79</v>
+      </c>
+      <c r="M10" s="175" t="s">
         <v>160</v>
       </c>
-      <c r="N8" s="209"/>
-      <c r="O8" s="209" t="s">
+      <c r="N10" s="175"/>
+      <c r="O10" s="175" t="s">
         <v>180</v>
       </c>
-      <c r="P8" s="209" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="9" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B9" s="209">
-        <v>3</v>
-      </c>
-      <c r="C9" s="209" t="s">
-        <v>175</v>
-      </c>
-      <c r="D9" s="209" t="s">
-        <v>174</v>
-      </c>
-      <c r="E9" s="209">
-        <v>1.98</v>
-      </c>
-      <c r="F9" s="209" t="s">
-        <v>173</v>
-      </c>
-      <c r="G9" s="209">
-        <v>4</v>
-      </c>
-      <c r="H9" s="210">
-        <v>45984</v>
-      </c>
-      <c r="I9" s="210">
-        <v>45976</v>
-      </c>
-      <c r="J9" s="210">
-        <v>45982</v>
-      </c>
-      <c r="K9" s="210">
-        <v>45984</v>
-      </c>
-      <c r="L9" s="209" t="s">
-        <v>178</v>
-      </c>
-      <c r="M9" s="209" t="s">
-        <v>160</v>
-      </c>
-      <c r="N9" s="209"/>
-      <c r="O9" s="209" t="s">
-        <v>182</v>
-      </c>
-      <c r="P9" s="209" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="10" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B10" s="209">
-        <v>4</v>
-      </c>
-      <c r="C10" s="209" t="s">
-        <v>176</v>
-      </c>
-      <c r="D10" s="209" t="s">
-        <v>177</v>
-      </c>
-      <c r="E10" s="209">
-        <v>2.46</v>
-      </c>
-      <c r="F10" s="209" t="s">
-        <v>173</v>
-      </c>
-      <c r="G10" s="209">
-        <v>5</v>
-      </c>
-      <c r="H10" s="210">
-        <v>45971</v>
-      </c>
-      <c r="I10" s="210">
-        <v>45984</v>
-      </c>
-      <c r="J10" s="210">
-        <v>45991</v>
-      </c>
-      <c r="K10" s="210">
-        <v>45993</v>
-      </c>
-      <c r="L10" s="209" t="s">
+      <c r="P10" s="175" t="s">
         <v>179</v>
-      </c>
-      <c r="M10" s="209" t="s">
-        <v>160</v>
-      </c>
-      <c r="N10" s="209"/>
-      <c r="O10" s="209" t="s">
-        <v>182</v>
-      </c>
-      <c r="P10" s="209" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.35">
@@ -6640,10 +6637,10 @@
       <c r="I11" s="127"/>
       <c r="J11" s="127"/>
       <c r="K11" s="173"/>
-      <c r="L11" s="209"/>
-      <c r="N11" s="209"/>
-      <c r="O11" s="209"/>
-      <c r="P11" s="209"/>
+      <c r="L11" s="175"/>
+      <c r="N11" s="175"/>
+      <c r="O11" s="175"/>
+      <c r="P11" s="175"/>
     </row>
     <row r="12" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B12" s="152"/>
@@ -6656,10 +6653,10 @@
       <c r="I12" s="92"/>
       <c r="J12" s="92"/>
       <c r="K12" s="155"/>
-      <c r="L12" s="209"/>
-      <c r="N12" s="209"/>
-      <c r="O12" s="209"/>
-      <c r="P12" s="209"/>
+      <c r="L12" s="175"/>
+      <c r="N12" s="175"/>
+      <c r="O12" s="175"/>
+      <c r="P12" s="175"/>
     </row>
     <row r="13" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="146"/>
@@ -6969,118 +6966,118 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="177" t="s">
+      <c r="A18" s="195" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="177" t="s">
+      <c r="B18" s="195" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="174" t="s">
+      <c r="C18" s="191" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="174" t="s">
+      <c r="D18" s="191" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="177" t="s">
+      <c r="E18" s="195" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="189" t="s">
+      <c r="F18" s="182" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="189"/>
-      <c r="H18" s="189"/>
-      <c r="I18" s="189"/>
-      <c r="J18" s="189"/>
-      <c r="K18" s="182" t="s">
+      <c r="G18" s="182"/>
+      <c r="H18" s="182"/>
+      <c r="I18" s="182"/>
+      <c r="J18" s="182"/>
+      <c r="K18" s="185" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="174" t="s">
+      <c r="M18" s="191" t="s">
         <v>36</v>
       </c>
-      <c r="O18" s="183" t="s">
+      <c r="O18" s="186" t="s">
         <v>31</v>
       </c>
-      <c r="P18" s="184"/>
-      <c r="Q18" s="184"/>
-      <c r="R18" s="184"/>
-      <c r="S18" s="184"/>
-      <c r="T18" s="185"/>
-      <c r="V18" s="183" t="s">
+      <c r="P18" s="187"/>
+      <c r="Q18" s="187"/>
+      <c r="R18" s="187"/>
+      <c r="S18" s="187"/>
+      <c r="T18" s="188"/>
+      <c r="V18" s="186" t="s">
         <v>30</v>
       </c>
-      <c r="W18" s="184"/>
-      <c r="X18" s="184"/>
-      <c r="Y18" s="184"/>
-      <c r="Z18" s="184"/>
-      <c r="AA18" s="185"/>
-      <c r="AB18" s="186" t="s">
+      <c r="W18" s="187"/>
+      <c r="X18" s="187"/>
+      <c r="Y18" s="187"/>
+      <c r="Z18" s="187"/>
+      <c r="AA18" s="188"/>
+      <c r="AB18" s="189" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="178"/>
-      <c r="B19" s="178"/>
-      <c r="C19" s="175"/>
-      <c r="D19" s="178"/>
-      <c r="E19" s="178"/>
-      <c r="F19" s="205" t="s">
+      <c r="A19" s="196"/>
+      <c r="B19" s="196"/>
+      <c r="C19" s="193"/>
+      <c r="D19" s="196"/>
+      <c r="E19" s="196"/>
+      <c r="F19" s="207" t="s">
         <v>40</v>
       </c>
-      <c r="G19" s="206" t="s">
+      <c r="G19" s="208" t="s">
         <v>44</v>
       </c>
-      <c r="H19" s="207"/>
-      <c r="I19" s="206" t="s">
+      <c r="H19" s="209"/>
+      <c r="I19" s="208" t="s">
         <v>45</v>
       </c>
-      <c r="J19" s="207"/>
-      <c r="K19" s="182"/>
-      <c r="M19" s="188"/>
-      <c r="O19" s="180" t="s">
+      <c r="J19" s="209"/>
+      <c r="K19" s="185"/>
+      <c r="M19" s="192"/>
+      <c r="O19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="P19" s="180" t="s">
+      <c r="P19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="Q19" s="180" t="s">
+      <c r="Q19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="R19" s="180" t="s">
+      <c r="R19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="S19" s="180" t="s">
+      <c r="S19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="T19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="180" t="s">
+      <c r="V19" s="183" t="s">
         <v>24</v>
       </c>
-      <c r="W19" s="180" t="s">
+      <c r="W19" s="183" t="s">
         <v>25</v>
       </c>
-      <c r="X19" s="180" t="s">
+      <c r="X19" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="Y19" s="180" t="s">
+      <c r="Y19" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="Z19" s="180" t="s">
+      <c r="Z19" s="183" t="s">
         <v>28</v>
       </c>
       <c r="AA19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AB19" s="187"/>
+      <c r="AB19" s="190"/>
     </row>
     <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="178"/>
-      <c r="B20" s="178"/>
-      <c r="C20" s="175"/>
-      <c r="D20" s="178"/>
-      <c r="E20" s="178"/>
-      <c r="F20" s="205"/>
+      <c r="A20" s="196"/>
+      <c r="B20" s="196"/>
+      <c r="C20" s="193"/>
+      <c r="D20" s="196"/>
+      <c r="E20" s="196"/>
+      <c r="F20" s="207"/>
       <c r="G20" s="93" t="s">
         <v>10</v>
       </c>
@@ -7099,17 +7096,17 @@
       <c r="M20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O20" s="181"/>
-      <c r="P20" s="181"/>
-      <c r="Q20" s="181"/>
-      <c r="R20" s="181"/>
-      <c r="S20" s="181"/>
+      <c r="O20" s="184"/>
+      <c r="P20" s="184"/>
+      <c r="Q20" s="184"/>
+      <c r="R20" s="184"/>
+      <c r="S20" s="184"/>
       <c r="T20" s="19"/>
-      <c r="V20" s="181"/>
-      <c r="W20" s="181"/>
-      <c r="X20" s="181"/>
-      <c r="Y20" s="181"/>
-      <c r="Z20" s="181"/>
+      <c r="V20" s="184"/>
+      <c r="W20" s="184"/>
+      <c r="X20" s="184"/>
+      <c r="Y20" s="184"/>
+      <c r="Z20" s="184"/>
       <c r="AA20" s="19" t="s">
         <v>20</v>
       </c>
@@ -7130,7 +7127,7 @@
       <c r="D21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="204" t="s">
+      <c r="E21" s="210" t="s">
         <v>98</v>
       </c>
       <c r="F21" s="113">
@@ -7204,7 +7201,7 @@
       <c r="D22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="204"/>
+      <c r="E22" s="210"/>
       <c r="F22" s="113">
         <v>45913</v>
       </c>
@@ -7276,7 +7273,7 @@
       <c r="D23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="204"/>
+      <c r="E23" s="210"/>
       <c r="F23" s="113">
         <v>45910</v>
       </c>
@@ -7348,7 +7345,7 @@
       <c r="D24" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="204"/>
+      <c r="E24" s="210"/>
       <c r="F24" s="113">
         <v>45927</v>
       </c>
@@ -7420,7 +7417,7 @@
       <c r="D25" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="204"/>
+      <c r="E25" s="210"/>
       <c r="F25" s="113">
         <v>45915</v>
       </c>
@@ -8115,6 +8112,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O18:T18"/>
+    <mergeCell ref="V18:AA18"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
     <mergeCell ref="AB18:AB19"/>
     <mergeCell ref="F19:F20"/>
     <mergeCell ref="G19:H19"/>
@@ -8128,18 +8137,6 @@
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
     <mergeCell ref="S19:S20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="O18:T18"/>
-    <mergeCell ref="V18:AA18"/>
-    <mergeCell ref="V19:V20"/>
   </mergeCells>
   <conditionalFormatting sqref="C26:C27">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="4DT6">

</xml_diff>

<commit_message>
Update binary files and enhance dashboard callbacks for project metrics
- Updated binary files including `ErectionCompiled_Output.xlsx`, `StringingCompiled_Output.xlsx`, and `Micro Plan - TA-418 Nov'25.xlsx` to reflect recent changes in data processing.
- Improved dashboard callback functions to enhance project metrics handling and UI interactions.
- Removed outdated button row in the modal layout for a cleaner interface.
</commit_message>
<xml_diff>
--- a/Raw Data/Micro Plans/November 2025/Micro Plan - TA-418 Nov'25.xlsx
+++ b/Raw Data/Micro Plans/November 2025/Micro Plan - TA-418 Nov'25.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaushikb\Documents\Work\Git\Office-work-\Raw Data\Micro Plans\November 2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF7DE310-4FF0-482E-8F1E-5B8361E39611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0DEBFE-D915-4FEA-B42A-46432A0B3DFE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="757" firstSheet="2" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1438,7 +1438,7 @@
     <xf numFmtId="164" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="164" fontId="31" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="211">
+  <cellXfs count="210">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1873,9 +1873,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1960,69 +1957,69 @@
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2050,6 +2047,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2057,9 +2057,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2775,6 +2772,31 @@
     </dxf>
     <dxf>
       <font>
+        <color indexed="20"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="45"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="20"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor indexed="45"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color indexed="20"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color indexed="17"/>
       </font>
       <fill>
@@ -2782,31 +2804,6 @@
           <bgColor indexed="42"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="45"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor indexed="45"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color indexed="20"/>
-      </font>
     </dxf>
     <dxf>
       <font>
@@ -3628,137 +3625,137 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:33" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="195" t="s">
+      <c r="A18" s="179" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="195" t="s">
+      <c r="B18" s="179" t="s">
         <v>5</v>
       </c>
-      <c r="C18" s="191" t="s">
+      <c r="C18" s="176" t="s">
         <v>6</v>
       </c>
-      <c r="D18" s="195" t="s">
+      <c r="D18" s="179" t="s">
         <v>7</v>
       </c>
-      <c r="E18" s="191" t="s">
+      <c r="E18" s="176" t="s">
         <v>16</v>
       </c>
-      <c r="F18" s="191" t="s">
+      <c r="F18" s="176" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="195" t="s">
+      <c r="G18" s="179" t="s">
         <v>8</v>
       </c>
-      <c r="H18" s="182" t="s">
+      <c r="H18" s="191" t="s">
         <v>18</v>
       </c>
-      <c r="I18" s="182"/>
-      <c r="J18" s="182"/>
-      <c r="K18" s="182"/>
-      <c r="L18" s="182"/>
-      <c r="M18" s="182"/>
-      <c r="N18" s="182"/>
-      <c r="O18" s="182"/>
-      <c r="P18" s="185" t="s">
+      <c r="I18" s="191"/>
+      <c r="J18" s="191"/>
+      <c r="K18" s="191"/>
+      <c r="L18" s="191"/>
+      <c r="M18" s="191"/>
+      <c r="N18" s="191"/>
+      <c r="O18" s="191"/>
+      <c r="P18" s="184" t="s">
         <v>19</v>
       </c>
-      <c r="R18" s="191" t="s">
+      <c r="R18" s="176" t="s">
         <v>36</v>
       </c>
-      <c r="T18" s="186" t="s">
+      <c r="T18" s="185" t="s">
         <v>31</v>
       </c>
-      <c r="U18" s="187"/>
-      <c r="V18" s="187"/>
-      <c r="W18" s="187"/>
-      <c r="X18" s="187"/>
-      <c r="Y18" s="188"/>
-      <c r="AA18" s="186" t="s">
+      <c r="U18" s="186"/>
+      <c r="V18" s="186"/>
+      <c r="W18" s="186"/>
+      <c r="X18" s="186"/>
+      <c r="Y18" s="187"/>
+      <c r="AA18" s="185" t="s">
         <v>30</v>
       </c>
-      <c r="AB18" s="187"/>
-      <c r="AC18" s="187"/>
-      <c r="AD18" s="187"/>
-      <c r="AE18" s="187"/>
-      <c r="AF18" s="188"/>
-      <c r="AG18" s="189" t="s">
+      <c r="AB18" s="186"/>
+      <c r="AC18" s="186"/>
+      <c r="AD18" s="186"/>
+      <c r="AE18" s="186"/>
+      <c r="AF18" s="187"/>
+      <c r="AG18" s="188" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:33" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="196"/>
-      <c r="B19" s="196"/>
-      <c r="C19" s="193"/>
-      <c r="D19" s="196"/>
-      <c r="E19" s="193"/>
-      <c r="F19" s="193"/>
-      <c r="G19" s="196"/>
-      <c r="H19" s="181" t="s">
+      <c r="A19" s="180"/>
+      <c r="B19" s="180"/>
+      <c r="C19" s="177"/>
+      <c r="D19" s="180"/>
+      <c r="E19" s="177"/>
+      <c r="F19" s="177"/>
+      <c r="G19" s="180"/>
+      <c r="H19" s="196" t="s">
         <v>9</v>
       </c>
-      <c r="I19" s="181"/>
-      <c r="J19" s="181" t="s">
+      <c r="I19" s="196"/>
+      <c r="J19" s="196" t="s">
         <v>12</v>
       </c>
-      <c r="K19" s="181"/>
-      <c r="L19" s="181" t="s">
+      <c r="K19" s="196"/>
+      <c r="L19" s="196" t="s">
         <v>13</v>
       </c>
-      <c r="M19" s="181"/>
-      <c r="N19" s="179" t="s">
+      <c r="M19" s="196"/>
+      <c r="N19" s="192" t="s">
         <v>15</v>
       </c>
-      <c r="O19" s="179" t="s">
+      <c r="O19" s="192" t="s">
         <v>14</v>
       </c>
-      <c r="P19" s="185"/>
-      <c r="R19" s="192"/>
-      <c r="T19" s="183" t="s">
+      <c r="P19" s="184"/>
+      <c r="R19" s="190"/>
+      <c r="T19" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="U19" s="183" t="s">
+      <c r="U19" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="V19" s="183" t="s">
+      <c r="V19" s="182" t="s">
         <v>26</v>
       </c>
-      <c r="W19" s="183" t="s">
+      <c r="W19" s="182" t="s">
         <v>27</v>
       </c>
-      <c r="X19" s="183" t="s">
+      <c r="X19" s="182" t="s">
         <v>28</v>
       </c>
       <c r="Y19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AA19" s="183" t="s">
+      <c r="AA19" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="AB19" s="183" t="s">
+      <c r="AB19" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="AC19" s="183" t="s">
+      <c r="AC19" s="182" t="s">
         <v>26</v>
       </c>
-      <c r="AD19" s="183" t="s">
+      <c r="AD19" s="182" t="s">
         <v>27</v>
       </c>
-      <c r="AE19" s="183" t="s">
+      <c r="AE19" s="182" t="s">
         <v>28</v>
       </c>
       <c r="AF19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AG19" s="190"/>
+      <c r="AG19" s="189"/>
     </row>
     <row r="20" spans="1:33" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="197"/>
-      <c r="B20" s="196"/>
-      <c r="C20" s="193"/>
-      <c r="D20" s="196"/>
-      <c r="E20" s="194"/>
-      <c r="F20" s="194"/>
-      <c r="G20" s="196"/>
+      <c r="A20" s="181"/>
+      <c r="B20" s="180"/>
+      <c r="C20" s="177"/>
+      <c r="D20" s="180"/>
+      <c r="E20" s="178"/>
+      <c r="F20" s="178"/>
+      <c r="G20" s="180"/>
       <c r="H20" s="93" t="s">
         <v>10</v>
       </c>
@@ -3777,25 +3774,25 @@
       <c r="M20" s="93" t="s">
         <v>11</v>
       </c>
-      <c r="N20" s="180"/>
-      <c r="O20" s="180"/>
+      <c r="N20" s="193"/>
+      <c r="O20" s="193"/>
       <c r="P20" s="44" t="s">
         <v>50</v>
       </c>
       <c r="R20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="T20" s="184"/>
-      <c r="U20" s="184"/>
-      <c r="V20" s="184"/>
-      <c r="W20" s="184"/>
-      <c r="X20" s="184"/>
+      <c r="T20" s="183"/>
+      <c r="U20" s="183"/>
+      <c r="V20" s="183"/>
+      <c r="W20" s="183"/>
+      <c r="X20" s="183"/>
       <c r="Y20" s="19"/>
-      <c r="AA20" s="184"/>
-      <c r="AB20" s="184"/>
-      <c r="AC20" s="184"/>
-      <c r="AD20" s="184"/>
-      <c r="AE20" s="184"/>
+      <c r="AA20" s="183"/>
+      <c r="AB20" s="183"/>
+      <c r="AC20" s="183"/>
+      <c r="AD20" s="183"/>
+      <c r="AE20" s="183"/>
       <c r="AF20" s="19" t="s">
         <v>50</v>
       </c>
@@ -4066,7 +4063,7 @@
       <c r="D25" s="85"/>
       <c r="E25" s="100"/>
       <c r="F25" s="8"/>
-      <c r="G25" s="177"/>
+      <c r="G25" s="194"/>
       <c r="H25" s="98"/>
       <c r="I25" s="98"/>
       <c r="J25" s="98"/>
@@ -4124,7 +4121,7 @@
       <c r="D26" s="8"/>
       <c r="E26" s="101"/>
       <c r="F26" s="96"/>
-      <c r="G26" s="178"/>
+      <c r="G26" s="195"/>
       <c r="H26" s="98"/>
       <c r="I26" s="98"/>
       <c r="J26" s="98"/>
@@ -4479,13 +4476,16 @@
     <filterColumn colId="13" showButton="0"/>
   </autoFilter>
   <mergeCells count="29">
-    <mergeCell ref="F18:F20"/>
-    <mergeCell ref="G18:G20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="O19:O20"/>
+    <mergeCell ref="H19:I19"/>
+    <mergeCell ref="J19:K19"/>
+    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="H18:O18"/>
+    <mergeCell ref="N19:N20"/>
+    <mergeCell ref="U19:U20"/>
+    <mergeCell ref="V19:V20"/>
+    <mergeCell ref="W19:W20"/>
     <mergeCell ref="X19:X20"/>
     <mergeCell ref="P18:P19"/>
     <mergeCell ref="AA18:AF18"/>
@@ -4498,16 +4498,13 @@
     <mergeCell ref="R18:R19"/>
     <mergeCell ref="T18:Y18"/>
     <mergeCell ref="T19:T20"/>
-    <mergeCell ref="H18:O18"/>
-    <mergeCell ref="N19:N20"/>
-    <mergeCell ref="U19:U20"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="O19:O20"/>
-    <mergeCell ref="H19:I19"/>
-    <mergeCell ref="J19:K19"/>
-    <mergeCell ref="L19:M19"/>
+    <mergeCell ref="F18:F20"/>
+    <mergeCell ref="G18:G20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
   </mergeCells>
   <phoneticPr fontId="8" type="noConversion"/>
   <conditionalFormatting sqref="B21">
@@ -4582,17 +4579,17 @@
     <cfRule type="expression" dxfId="58" priority="1243" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$123, B26)+COUNTIF($D$142:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="57" priority="1245" stopIfTrue="1">
+    <cfRule type="expression" dxfId="57" priority="1244" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="56" priority="1246" stopIfTrue="1">
+    <cfRule type="expression" dxfId="56" priority="1245" stopIfTrue="1">
       <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="55" priority="1247" stopIfTrue="1">
+    <cfRule type="expression" dxfId="55" priority="1246" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="54" priority="1247" stopIfTrue="1">
       <formula>AND(COUNTIF($D$474:$D$65380, B26)+COUNTIF($D$454:$D$455, B26)+COUNTIF($D$416:$D$417, B26)+COUNTIF($D$374:$D$377, B26)+COUNTIF($D$351:$D$352, B26)+COUNTIF($D$324:$D$325, B26)+COUNTIF($D$303:$D$303, B26)+COUNTIF($D$288:$D$289, B26)+COUNTIF($D$263:$D$263, B26)+COUNTIF($D$252:$D$253, B26)+COUNTIF($D$233:$D$234, B26)+COUNTIF($D$51:$D$218, B26)+COUNTIF($D$219:$D$220, B26)+COUNTIF($D$1:$D$50, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="54" priority="1244" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$1:$D$191, B26)+COUNTIF($D$214:$D$65380, B26)&gt;1,NOT(ISBLANK(B26)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="B27">
@@ -4609,55 +4606,55 @@
     <cfRule type="duplicateValues" dxfId="47" priority="347"/>
   </conditionalFormatting>
   <conditionalFormatting sqref="L4">
-    <cfRule type="expression" dxfId="46" priority="1221" stopIfTrue="1">
+    <cfRule type="expression" dxfId="46" priority="1220" stopIfTrue="1">
+      <formula>AND(COUNTIF($C$314:$C$65460, L4)+COUNTIF($C$294:$C$295, L4)+COUNTIF($C$256:$C$257, L4)+COUNTIF($C$214:$C$217, L4)+COUNTIF($C$191:$C$192, L4)+COUNTIF($C$164:$C$165, L4)+COUNTIF($C$143:$C$143, L4)+COUNTIF($C$128:$C$129, L4)+COUNTIF($C$103:$C$103, L4)+COUNTIF($C$92:$C$93, L4)+COUNTIF($C$73:$C$74, L4)+COUNTIF($C$29:$C$56, L4)+COUNTIF($C$58:$C$60, L4)+COUNTIF($C$1:$C$27, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="45" priority="1221" stopIfTrue="1">
       <formula>AND(COUNTIF($C$1:$C$65460, L4)+COUNTIF(#REF!, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="45" priority="1220" stopIfTrue="1">
-      <formula>AND(COUNTIF($C$314:$C$65460, L4)+COUNTIF($C$294:$C$295, L4)+COUNTIF($C$256:$C$257, L4)+COUNTIF($C$214:$C$217, L4)+COUNTIF($C$191:$C$192, L4)+COUNTIF($C$164:$C$165, L4)+COUNTIF($C$143:$C$143, L4)+COUNTIF($C$128:$C$129, L4)+COUNTIF($C$103:$C$103, L4)+COUNTIF($C$92:$C$93, L4)+COUNTIF($C$73:$C$74, L4)+COUNTIF($C$29:$C$56, L4)+COUNTIF($C$58:$C$60, L4)+COUNTIF($C$1:$C$27, L4)&gt;1,NOT(ISBLANK(L4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M4">
-    <cfRule type="expression" dxfId="44" priority="1223" stopIfTrue="1">
+    <cfRule type="expression" dxfId="44" priority="1222" stopIfTrue="1">
+      <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="43" priority="1223" stopIfTrue="1">
       <formula>AND(COUNTIF($D$314:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="43" priority="1224" stopIfTrue="1">
+    <cfRule type="expression" dxfId="42" priority="1224" stopIfTrue="1">
       <formula>AND(COUNTIF($D$294:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="42" priority="1225" stopIfTrue="1">
+    <cfRule type="expression" dxfId="41" priority="1225" stopIfTrue="1">
       <formula>AND(COUNTIF($D$256:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="41" priority="1226" stopIfTrue="1">
+    <cfRule type="expression" dxfId="40" priority="1226" stopIfTrue="1">
       <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="40" priority="1227" stopIfTrue="1">
+    <cfRule type="expression" dxfId="39" priority="1227" stopIfTrue="1">
       <formula>AND(COUNTIF($D$214:$D$65460, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="39" priority="1228" stopIfTrue="1">
+    <cfRule type="expression" dxfId="38" priority="1228" stopIfTrue="1">
       <formula>AND(COUNTIF($D$191:$D$65460, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$51:$D$51, M4)+COUNTIF($D$53:$D$60, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="38" priority="1229" stopIfTrue="1">
+    <cfRule type="expression" dxfId="37" priority="1229" stopIfTrue="1">
       <formula>AND(COUNTIF($F$369:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$352:$F$353, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="37" priority="1230" stopIfTrue="1">
+    <cfRule type="expression" dxfId="36" priority="1230" stopIfTrue="1">
       <formula>AND(COUNTIF($F$352:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$332:$F$333, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="36" priority="1231" stopIfTrue="1">
+    <cfRule type="expression" dxfId="35" priority="1231" stopIfTrue="1">
       <formula>AND(COUNTIF($F$332:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$294:$F$295, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="35" priority="1232" stopIfTrue="1">
+    <cfRule type="expression" dxfId="34" priority="1232" stopIfTrue="1">
       <formula>AND(COUNTIF($F$294:$F$65454, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$252:$F$255, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="34" priority="1233" stopIfTrue="1">
+    <cfRule type="expression" dxfId="33" priority="1233" stopIfTrue="1">
       <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$96:$F$98, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="33" priority="1234" stopIfTrue="1">
+    <cfRule type="expression" dxfId="32" priority="1234" stopIfTrue="1">
       <formula>AND(COUNTIF($F$252:$F$65454, M4)+COUNTIF($F$229:$F$230, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="32" priority="1235" stopIfTrue="1">
+    <cfRule type="expression" dxfId="31" priority="1235" stopIfTrue="1">
       <formula>AND(COUNTIF($F$229:$F$65454, M4)+COUNTIF($F$202:$F$203, M4)+COUNTIF($F$181:$F$181, M4)+COUNTIF($F$166:$F$167, M4)+COUNTIF($F$1:$F$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$141:$F$141, M4)+COUNTIF($F$130:$F$131, M4)+COUNTIF(#REF!, M4)+COUNTIF($F$111:$F$112, M4)+COUNTIF($F$89:$F$89, M4)+COUNTIF($F$91:$F$98, M4)+COUNTIF(#REF!, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="31" priority="1222" stopIfTrue="1">
-      <formula>AND(COUNTIF($D$331:$D$65460, M4)+COUNTIF($D$1:$D$27, M4)+COUNTIF(#REF!, M4)+COUNTIF($D$314:$D$315, M4)+COUNTIF($D$294:$D$295, M4)+COUNTIF($D$256:$D$257, M4)+COUNTIF($D$214:$D$217, M4)+COUNTIF($D$191:$D$192, M4)+COUNTIF($D$164:$D$165, M4)+COUNTIF($D$143:$D$143, M4)+COUNTIF($D$128:$D$129, M4)+COUNTIF($D$103:$D$103, M4)+COUNTIF($D$92:$D$93, M4)+COUNTIF($D$73:$D$74, M4)+COUNTIF($D$58:$D$60, M4)&gt;1,NOT(ISBLANK(M4)))</formula>
     </cfRule>
   </conditionalFormatting>
   <printOptions horizontalCentered="1"/>
@@ -4778,7 +4775,7 @@
       <c r="Q4" s="70">
         <v>0</v>
       </c>
-      <c r="R4" s="198" t="s">
+      <c r="R4" s="197" t="s">
         <v>75</v>
       </c>
     </row>
@@ -4821,14 +4818,14 @@
       <c r="Q5" s="70">
         <v>0</v>
       </c>
-      <c r="R5" s="199"/>
+      <c r="R5" s="198"/>
     </row>
     <row r="6" spans="2:18" s="75" customFormat="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="200" t="s">
+      <c r="B6" s="199" t="s">
         <v>29</v>
       </c>
-      <c r="C6" s="201"/>
-      <c r="D6" s="202"/>
+      <c r="C6" s="200"/>
+      <c r="D6" s="201"/>
       <c r="E6" s="73">
         <v>160</v>
       </c>
@@ -4903,49 +4900,49 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:37" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="A1" s="160" t="s">
+      <c r="A1" s="159" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="160" t="s">
+      <c r="B1" s="159" t="s">
         <v>111</v>
       </c>
-      <c r="C1" s="159" t="s">
+      <c r="C1" s="158" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="159" t="s">
+      <c r="D1" s="158" t="s">
         <v>107</v>
       </c>
-      <c r="E1" s="160" t="s">
+      <c r="E1" s="159" t="s">
         <v>108</v>
       </c>
-      <c r="F1" s="160" t="s">
+      <c r="F1" s="159" t="s">
         <v>103</v>
       </c>
-      <c r="G1" s="159" t="s">
+      <c r="G1" s="158" t="s">
         <v>104</v>
       </c>
-      <c r="H1" s="160" t="s">
+      <c r="H1" s="159" t="s">
         <v>105</v>
       </c>
-      <c r="I1" s="159" t="s">
+      <c r="I1" s="158" t="s">
         <v>106</v>
       </c>
-      <c r="J1" s="161" t="s">
+      <c r="J1" s="160" t="s">
         <v>112</v>
       </c>
-      <c r="K1" s="168" t="s">
+      <c r="K1" s="167" t="s">
         <v>109</v>
       </c>
-      <c r="L1" s="168" t="s">
+      <c r="L1" s="167" t="s">
         <v>110</v>
       </c>
-      <c r="M1" s="161" t="s">
+      <c r="M1" s="160" t="s">
         <v>38</v>
       </c>
-      <c r="N1" s="161" t="s">
+      <c r="N1" s="160" t="s">
         <v>39</v>
       </c>
-      <c r="O1" s="167" t="s">
+      <c r="O1" s="166" t="s">
         <v>161</v>
       </c>
       <c r="P1" s="126" t="s">
@@ -4956,7 +4953,7 @@
       <c r="A2" s="128">
         <v>1</v>
       </c>
-      <c r="B2" s="162" t="s">
+      <c r="B2" s="161" t="s">
         <v>120</v>
       </c>
       <c r="C2" s="8" t="s">
@@ -4965,7 +4962,7 @@
       <c r="D2" s="8">
         <v>89.028999999999996</v>
       </c>
-      <c r="E2" s="169" t="s">
+      <c r="E2" s="168" t="s">
         <v>150</v>
       </c>
       <c r="F2" s="129">
@@ -4978,14 +4975,14 @@
         <v>155</v>
       </c>
       <c r="I2" s="130"/>
-      <c r="J2" s="164">
+      <c r="J2" s="163">
         <v>45946</v>
       </c>
-      <c r="K2" s="165">
+      <c r="K2" s="164">
         <f>J2+3</f>
         <v>45949</v>
       </c>
-      <c r="L2" s="165">
+      <c r="L2" s="164">
         <v>45967</v>
       </c>
       <c r="M2" s="131">
@@ -4996,7 +4993,7 @@
         <f>M2+1</f>
         <v>45969</v>
       </c>
-      <c r="O2" s="166">
+      <c r="O2" s="165">
         <v>1150500</v>
       </c>
     </row>
@@ -5004,7 +5001,7 @@
       <c r="A3" s="128">
         <v>2</v>
       </c>
-      <c r="B3" s="163" t="s">
+      <c r="B3" s="162" t="s">
         <v>122</v>
       </c>
       <c r="C3" s="8" t="s">
@@ -5013,7 +5010,7 @@
       <c r="D3" s="8">
         <v>29.122</v>
       </c>
-      <c r="E3" s="169" t="s">
+      <c r="E3" s="168" t="s">
         <v>150</v>
       </c>
       <c r="F3" s="129">
@@ -5026,14 +5023,14 @@
         <v>155</v>
       </c>
       <c r="I3" s="130"/>
-      <c r="J3" s="164">
+      <c r="J3" s="163">
         <v>45966</v>
       </c>
-      <c r="K3" s="165">
+      <c r="K3" s="164">
         <f>J3+1</f>
         <v>45967</v>
       </c>
-      <c r="L3" s="165">
+      <c r="L3" s="164">
         <v>45971</v>
       </c>
       <c r="M3" s="131">
@@ -5044,7 +5041,7 @@
         <f t="shared" si="0"/>
         <v>45973</v>
       </c>
-      <c r="O3" s="166">
+      <c r="O3" s="165">
         <v>360000</v>
       </c>
       <c r="Q3" s="134"/>
@@ -5068,7 +5065,7 @@
       <c r="A4" s="128">
         <v>3</v>
       </c>
-      <c r="B4" s="163" t="s">
+      <c r="B4" s="162" t="s">
         <v>124</v>
       </c>
       <c r="C4" s="8" t="s">
@@ -5077,7 +5074,7 @@
       <c r="D4" s="8">
         <v>27.963000000000001</v>
       </c>
-      <c r="E4" s="169" t="s">
+      <c r="E4" s="168" t="s">
         <v>150</v>
       </c>
       <c r="F4" s="129">
@@ -5090,14 +5087,14 @@
         <v>155</v>
       </c>
       <c r="I4" s="130"/>
-      <c r="J4" s="164">
+      <c r="J4" s="163">
         <v>45971</v>
       </c>
-      <c r="K4" s="165">
+      <c r="K4" s="164">
         <f t="shared" ref="K4:K21" si="1">J4+1</f>
         <v>45972</v>
       </c>
-      <c r="L4" s="165">
+      <c r="L4" s="164">
         <v>45975</v>
       </c>
       <c r="M4" s="131">
@@ -5108,7 +5105,7 @@
         <f t="shared" si="0"/>
         <v>45977</v>
       </c>
-      <c r="O4" s="166">
+      <c r="O4" s="165">
         <v>308000</v>
       </c>
       <c r="Q4" s="137"/>
@@ -5132,7 +5129,7 @@
       <c r="A5" s="128">
         <v>4</v>
       </c>
-      <c r="B5" s="163" t="s">
+      <c r="B5" s="162" t="s">
         <v>126</v>
       </c>
       <c r="C5" s="8" t="s">
@@ -5141,7 +5138,7 @@
       <c r="D5" s="8">
         <v>26.846</v>
       </c>
-      <c r="E5" s="169" t="s">
+      <c r="E5" s="168" t="s">
         <v>150</v>
       </c>
       <c r="F5" s="129">
@@ -5154,14 +5151,14 @@
         <v>155</v>
       </c>
       <c r="I5" s="130"/>
-      <c r="J5" s="164">
+      <c r="J5" s="163">
         <v>45975</v>
       </c>
-      <c r="K5" s="165">
+      <c r="K5" s="164">
         <f t="shared" si="1"/>
         <v>45976</v>
       </c>
-      <c r="L5" s="165">
+      <c r="L5" s="164">
         <v>45979</v>
       </c>
       <c r="M5" s="131">
@@ -5172,7 +5169,7 @@
         <f t="shared" si="0"/>
         <v>45981</v>
       </c>
-      <c r="O5" s="166">
+      <c r="O5" s="165">
         <v>295000</v>
       </c>
       <c r="Q5" s="138"/>
@@ -5196,7 +5193,7 @@
       <c r="A6" s="128">
         <v>5</v>
       </c>
-      <c r="B6" s="163" t="s">
+      <c r="B6" s="162" t="s">
         <v>128</v>
       </c>
       <c r="C6" s="8" t="s">
@@ -5205,7 +5202,7 @@
       <c r="D6" s="8">
         <v>27.963000000000001</v>
       </c>
-      <c r="E6" s="169" t="s">
+      <c r="E6" s="168" t="s">
         <v>150</v>
       </c>
       <c r="F6" s="129">
@@ -5218,14 +5215,14 @@
         <v>155</v>
       </c>
       <c r="I6" s="130"/>
-      <c r="J6" s="164">
+      <c r="J6" s="163">
         <v>45979</v>
       </c>
-      <c r="K6" s="165">
+      <c r="K6" s="164">
         <f t="shared" si="1"/>
         <v>45980</v>
       </c>
-      <c r="L6" s="165">
+      <c r="L6" s="164">
         <v>45984</v>
       </c>
       <c r="M6" s="131">
@@ -5236,7 +5233,7 @@
         <f t="shared" si="0"/>
         <v>45986</v>
       </c>
-      <c r="O6" s="166">
+      <c r="O6" s="165">
         <v>308000</v>
       </c>
       <c r="Q6" s="138"/>
@@ -5260,7 +5257,7 @@
       <c r="A7" s="128">
         <v>6</v>
       </c>
-      <c r="B7" s="163" t="s">
+      <c r="B7" s="162" t="s">
         <v>81</v>
       </c>
       <c r="C7" s="8" t="s">
@@ -5269,7 +5266,7 @@
       <c r="D7" s="8">
         <v>73.176000000000002</v>
       </c>
-      <c r="E7" s="169" t="s">
+      <c r="E7" s="168" t="s">
         <v>150</v>
       </c>
       <c r="F7" s="129">
@@ -5282,14 +5279,14 @@
         <v>155</v>
       </c>
       <c r="I7" s="130"/>
-      <c r="J7" s="164">
+      <c r="J7" s="163">
         <v>45984</v>
       </c>
-      <c r="K7" s="165">
+      <c r="K7" s="164">
         <f t="shared" si="1"/>
         <v>45985</v>
       </c>
-      <c r="L7" s="165">
+      <c r="L7" s="164">
         <v>45991</v>
       </c>
       <c r="M7" s="131">
@@ -5300,7 +5297,7 @@
         <f t="shared" si="0"/>
         <v>45993</v>
       </c>
-      <c r="O7" s="166">
+      <c r="O7" s="165">
         <v>809000</v>
       </c>
       <c r="Q7" s="138"/>
@@ -5324,7 +5321,7 @@
       <c r="A8" s="128">
         <v>7</v>
       </c>
-      <c r="B8" s="163" t="s">
+      <c r="B8" s="162" t="s">
         <v>130</v>
       </c>
       <c r="C8" s="8" t="s">
@@ -5333,7 +5330,7 @@
       <c r="D8" s="8">
         <v>26.846</v>
       </c>
-      <c r="E8" s="169" t="s">
+      <c r="E8" s="168" t="s">
         <v>151</v>
       </c>
       <c r="F8" s="129">
@@ -5346,14 +5343,14 @@
         <v>154</v>
       </c>
       <c r="I8" s="130"/>
-      <c r="J8" s="164">
+      <c r="J8" s="163">
         <v>45959</v>
       </c>
-      <c r="K8" s="165">
+      <c r="K8" s="164">
         <f t="shared" si="1"/>
         <v>45960</v>
       </c>
-      <c r="L8" s="165">
+      <c r="L8" s="164">
         <v>45966</v>
       </c>
       <c r="M8" s="131">
@@ -5364,7 +5361,7 @@
         <f t="shared" si="0"/>
         <v>45968</v>
       </c>
-      <c r="O8" s="166">
+      <c r="O8" s="165">
         <v>295000</v>
       </c>
       <c r="Q8" s="138"/>
@@ -5388,7 +5385,7 @@
       <c r="A9" s="128">
         <v>8</v>
       </c>
-      <c r="B9" s="163" t="s">
+      <c r="B9" s="162" t="s">
         <v>131</v>
       </c>
       <c r="C9" s="8" t="s">
@@ -5397,7 +5394,7 @@
       <c r="D9" s="8">
         <v>27.963000000000001</v>
       </c>
-      <c r="E9" s="169" t="s">
+      <c r="E9" s="168" t="s">
         <v>151</v>
       </c>
       <c r="F9" s="129">
@@ -5410,14 +5407,14 @@
         <v>154</v>
       </c>
       <c r="I9" s="130"/>
-      <c r="J9" s="164">
+      <c r="J9" s="163">
         <v>45966</v>
       </c>
-      <c r="K9" s="165">
+      <c r="K9" s="164">
         <f t="shared" si="1"/>
         <v>45967</v>
       </c>
-      <c r="L9" s="165">
+      <c r="L9" s="164">
         <v>45971</v>
       </c>
       <c r="M9" s="131">
@@ -5428,7 +5425,7 @@
         <f t="shared" si="0"/>
         <v>45973</v>
       </c>
-      <c r="O9" s="166">
+      <c r="O9" s="165">
         <v>308000</v>
       </c>
       <c r="Q9" s="138"/>
@@ -5452,7 +5449,7 @@
       <c r="A10" s="128">
         <v>9</v>
       </c>
-      <c r="B10" s="163" t="s">
+      <c r="B10" s="162" t="s">
         <v>132</v>
       </c>
       <c r="C10" s="8" t="s">
@@ -5461,7 +5458,7 @@
       <c r="D10" s="8">
         <v>27.600999999999999</v>
       </c>
-      <c r="E10" s="169" t="s">
+      <c r="E10" s="168" t="s">
         <v>151</v>
       </c>
       <c r="F10" s="129">
@@ -5474,14 +5471,14 @@
         <v>154</v>
       </c>
       <c r="I10" s="130"/>
-      <c r="J10" s="164">
+      <c r="J10" s="163">
         <v>45972</v>
       </c>
-      <c r="K10" s="165">
+      <c r="K10" s="164">
         <f t="shared" si="1"/>
         <v>45973</v>
       </c>
-      <c r="L10" s="165">
+      <c r="L10" s="164">
         <v>45977</v>
       </c>
       <c r="M10" s="131">
@@ -5492,7 +5489,7 @@
         <f t="shared" si="0"/>
         <v>45979</v>
       </c>
-      <c r="O10" s="166">
+      <c r="O10" s="165">
         <v>304000</v>
       </c>
       <c r="Q10" s="138"/>
@@ -5517,7 +5514,7 @@
       <c r="A11" s="128">
         <v>10</v>
       </c>
-      <c r="B11" s="163" t="s">
+      <c r="B11" s="162" t="s">
         <v>134</v>
       </c>
       <c r="C11" s="8" t="s">
@@ -5526,7 +5523,7 @@
       <c r="D11" s="8">
         <v>26.846</v>
       </c>
-      <c r="E11" s="169" t="s">
+      <c r="E11" s="168" t="s">
         <v>151</v>
       </c>
       <c r="F11" s="129">
@@ -5539,14 +5536,14 @@
         <v>154</v>
       </c>
       <c r="I11" s="130"/>
-      <c r="J11" s="164">
+      <c r="J11" s="163">
         <v>45977</v>
       </c>
-      <c r="K11" s="165">
+      <c r="K11" s="164">
         <f t="shared" si="1"/>
         <v>45978</v>
       </c>
-      <c r="L11" s="165">
+      <c r="L11" s="164">
         <v>45982</v>
       </c>
       <c r="M11" s="131">
@@ -5557,7 +5554,7 @@
         <f t="shared" si="0"/>
         <v>45984</v>
       </c>
-      <c r="O11" s="166">
+      <c r="O11" s="165">
         <v>295000</v>
       </c>
       <c r="Q11" s="138"/>
@@ -5581,7 +5578,7 @@
       <c r="A12" s="128">
         <v>11</v>
       </c>
-      <c r="B12" s="163" t="s">
+      <c r="B12" s="162" t="s">
         <v>135</v>
       </c>
       <c r="C12" s="8" t="s">
@@ -5590,7 +5587,7 @@
       <c r="D12" s="8">
         <v>45.136000000000003</v>
       </c>
-      <c r="E12" s="169" t="s">
+      <c r="E12" s="168" t="s">
         <v>151</v>
       </c>
       <c r="F12" s="129">
@@ -5603,14 +5600,14 @@
         <v>154</v>
       </c>
       <c r="I12" s="130"/>
-      <c r="J12" s="164">
+      <c r="J12" s="163">
         <v>45983</v>
       </c>
-      <c r="K12" s="165">
+      <c r="K12" s="164">
         <f t="shared" si="1"/>
         <v>45984</v>
       </c>
-      <c r="L12" s="165">
+      <c r="L12" s="164">
         <v>45990</v>
       </c>
       <c r="M12" s="131">
@@ -5621,7 +5618,7 @@
         <f t="shared" si="0"/>
         <v>45992</v>
       </c>
-      <c r="O12" s="166">
+      <c r="O12" s="165">
         <v>488000</v>
       </c>
       <c r="Q12" s="138"/>
@@ -5645,7 +5642,7 @@
       <c r="A13" s="128">
         <v>12</v>
       </c>
-      <c r="B13" s="163" t="s">
+      <c r="B13" s="162" t="s">
         <v>137</v>
       </c>
       <c r="C13" s="8" t="s">
@@ -5654,7 +5651,7 @@
       <c r="D13" s="8">
         <v>89.028999999999996</v>
       </c>
-      <c r="E13" s="169" t="s">
+      <c r="E13" s="168" t="s">
         <v>152</v>
       </c>
       <c r="F13" s="129">
@@ -5667,14 +5664,14 @@
         <v>156</v>
       </c>
       <c r="I13" s="130"/>
-      <c r="J13" s="164">
+      <c r="J13" s="163">
         <v>45946</v>
       </c>
-      <c r="K13" s="165">
+      <c r="K13" s="164">
         <f>J13+3</f>
         <v>45949</v>
       </c>
-      <c r="L13" s="165">
+      <c r="L13" s="164">
         <v>45968</v>
       </c>
       <c r="M13" s="131">
@@ -5685,7 +5682,7 @@
         <f t="shared" si="0"/>
         <v>45970</v>
       </c>
-      <c r="O13" s="166">
+      <c r="O13" s="165">
         <v>1151000</v>
       </c>
       <c r="Q13" s="138"/>
@@ -5709,7 +5706,7 @@
       <c r="A14" s="128">
         <v>13</v>
       </c>
-      <c r="B14" s="163" t="s">
+      <c r="B14" s="162" t="s">
         <v>138</v>
       </c>
       <c r="C14" s="8" t="s">
@@ -5718,7 +5715,7 @@
       <c r="D14" s="8">
         <v>51.673000000000002</v>
       </c>
-      <c r="E14" s="169" t="s">
+      <c r="E14" s="168" t="s">
         <v>152</v>
       </c>
       <c r="F14" s="129">
@@ -5731,14 +5728,14 @@
         <v>156</v>
       </c>
       <c r="I14" s="130"/>
-      <c r="J14" s="164">
+      <c r="J14" s="163">
         <v>45968</v>
       </c>
-      <c r="K14" s="165">
+      <c r="K14" s="164">
         <f t="shared" si="1"/>
         <v>45969</v>
       </c>
-      <c r="L14" s="165">
+      <c r="L14" s="164">
         <v>45975</v>
       </c>
       <c r="M14" s="131">
@@ -5749,7 +5746,7 @@
         <f t="shared" si="0"/>
         <v>45977</v>
       </c>
-      <c r="O14" s="166">
+      <c r="O14" s="165">
         <v>562000</v>
       </c>
       <c r="Q14" s="138"/>
@@ -5773,7 +5770,7 @@
       <c r="A15" s="128">
         <v>14</v>
       </c>
-      <c r="B15" s="163" t="s">
+      <c r="B15" s="162" t="s">
         <v>140</v>
       </c>
       <c r="C15" s="8" t="s">
@@ -5782,7 +5779,7 @@
       <c r="D15" s="8">
         <v>29.122</v>
       </c>
-      <c r="E15" s="169" t="s">
+      <c r="E15" s="168" t="s">
         <v>152</v>
       </c>
       <c r="F15" s="129">
@@ -5795,14 +5792,14 @@
         <v>156</v>
       </c>
       <c r="I15" s="130"/>
-      <c r="J15" s="164">
+      <c r="J15" s="163">
         <v>45975</v>
       </c>
-      <c r="K15" s="165">
+      <c r="K15" s="164">
         <f t="shared" si="1"/>
         <v>45976</v>
       </c>
-      <c r="L15" s="165">
+      <c r="L15" s="164">
         <v>45980</v>
       </c>
       <c r="M15" s="131">
@@ -5813,7 +5810,7 @@
         <f t="shared" si="0"/>
         <v>45982</v>
       </c>
-      <c r="O15" s="166">
+      <c r="O15" s="165">
         <v>360000</v>
       </c>
       <c r="Q15" s="138"/>
@@ -5837,7 +5834,7 @@
       <c r="A16" s="128">
         <v>15</v>
       </c>
-      <c r="B16" s="163" t="s">
+      <c r="B16" s="162" t="s">
         <v>141</v>
       </c>
       <c r="C16" s="8" t="s">
@@ -5846,7 +5843,7 @@
       <c r="D16" s="8">
         <v>26.846</v>
       </c>
-      <c r="E16" s="169" t="s">
+      <c r="E16" s="168" t="s">
         <v>152</v>
       </c>
       <c r="F16" s="129">
@@ -5859,14 +5856,14 @@
         <v>156</v>
       </c>
       <c r="I16" s="130"/>
-      <c r="J16" s="164">
+      <c r="J16" s="163">
         <v>45980</v>
       </c>
-      <c r="K16" s="165">
+      <c r="K16" s="164">
         <f t="shared" si="1"/>
         <v>45981</v>
       </c>
-      <c r="L16" s="165">
+      <c r="L16" s="164">
         <v>45985</v>
       </c>
       <c r="M16" s="131">
@@ -5877,7 +5874,7 @@
         <f t="shared" si="0"/>
         <v>45987</v>
       </c>
-      <c r="O16" s="166">
+      <c r="O16" s="165">
         <v>295000</v>
       </c>
       <c r="Q16" s="138"/>
@@ -5901,7 +5898,7 @@
       <c r="A17" s="128">
         <v>16</v>
       </c>
-      <c r="B17" s="162" t="s">
+      <c r="B17" s="161" t="s">
         <v>142</v>
       </c>
       <c r="C17" s="8" t="s">
@@ -5910,7 +5907,7 @@
       <c r="D17" s="8">
         <v>26.846</v>
       </c>
-      <c r="E17" s="169" t="s">
+      <c r="E17" s="168" t="s">
         <v>152</v>
       </c>
       <c r="F17" s="129">
@@ -5923,14 +5920,14 @@
         <v>156</v>
       </c>
       <c r="I17" s="130"/>
-      <c r="J17" s="164">
+      <c r="J17" s="163">
         <v>45985</v>
       </c>
-      <c r="K17" s="165">
+      <c r="K17" s="164">
         <f t="shared" si="1"/>
         <v>45986</v>
       </c>
-      <c r="L17" s="165">
+      <c r="L17" s="164">
         <v>45990</v>
       </c>
       <c r="M17" s="131">
@@ -5941,7 +5938,7 @@
         <f t="shared" si="0"/>
         <v>45992</v>
       </c>
-      <c r="O17" s="166">
+      <c r="O17" s="165">
         <v>295000</v>
       </c>
       <c r="Q17" s="138"/>
@@ -5965,7 +5962,7 @@
       <c r="A18" s="128">
         <v>17</v>
       </c>
-      <c r="B18" s="162" t="s">
+      <c r="B18" s="161" t="s">
         <v>143</v>
       </c>
       <c r="C18" s="8" t="s">
@@ -5974,7 +5971,7 @@
       <c r="D18" s="8">
         <v>26.846</v>
       </c>
-      <c r="E18" s="169" t="s">
+      <c r="E18" s="168" t="s">
         <v>144</v>
       </c>
       <c r="F18" s="129">
@@ -5987,14 +5984,14 @@
         <v>157</v>
       </c>
       <c r="I18" s="130"/>
-      <c r="J18" s="164">
+      <c r="J18" s="163">
         <v>45969</v>
       </c>
-      <c r="K18" s="165">
+      <c r="K18" s="164">
         <f t="shared" si="1"/>
         <v>45970</v>
       </c>
-      <c r="L18" s="165">
+      <c r="L18" s="164">
         <v>45974</v>
       </c>
       <c r="M18" s="131">
@@ -6005,7 +6002,7 @@
         <f t="shared" si="0"/>
         <v>45976</v>
       </c>
-      <c r="O18" s="166">
+      <c r="O18" s="165">
         <v>295000</v>
       </c>
       <c r="Q18" s="138"/>
@@ -6029,7 +6026,7 @@
       <c r="A19" s="128">
         <v>18</v>
       </c>
-      <c r="B19" s="162" t="s">
+      <c r="B19" s="161" t="s">
         <v>145</v>
       </c>
       <c r="C19" s="8" t="s">
@@ -6038,7 +6035,7 @@
       <c r="D19" s="8">
         <v>33.304000000000002</v>
       </c>
-      <c r="E19" s="169" t="s">
+      <c r="E19" s="168" t="s">
         <v>144</v>
       </c>
       <c r="F19" s="129">
@@ -6054,11 +6051,11 @@
       <c r="J19" s="113">
         <v>45974</v>
       </c>
-      <c r="K19" s="165">
+      <c r="K19" s="164">
         <f t="shared" si="1"/>
         <v>45975</v>
       </c>
-      <c r="L19" s="165">
+      <c r="L19" s="164">
         <v>45979</v>
       </c>
       <c r="M19" s="131">
@@ -6069,7 +6066,7 @@
         <f t="shared" si="0"/>
         <v>45981</v>
       </c>
-      <c r="O19" s="166">
+      <c r="O19" s="165">
         <v>374000</v>
       </c>
       <c r="Q19" s="138"/>
@@ -6093,7 +6090,7 @@
       <c r="A20" s="128">
         <v>19</v>
       </c>
-      <c r="B20" s="162" t="s">
+      <c r="B20" s="161" t="s">
         <v>147</v>
       </c>
       <c r="C20" s="8" t="s">
@@ -6102,7 +6099,7 @@
       <c r="D20" s="8">
         <v>26.846</v>
       </c>
-      <c r="E20" s="169" t="s">
+      <c r="E20" s="168" t="s">
         <v>144</v>
       </c>
       <c r="F20" s="129">
@@ -6118,11 +6115,11 @@
       <c r="J20" s="113">
         <v>45979</v>
       </c>
-      <c r="K20" s="165">
+      <c r="K20" s="164">
         <f t="shared" si="1"/>
         <v>45980</v>
       </c>
-      <c r="L20" s="165">
+      <c r="L20" s="164">
         <v>45984</v>
       </c>
       <c r="M20" s="131">
@@ -6133,7 +6130,7 @@
         <f t="shared" si="0"/>
         <v>45986</v>
       </c>
-      <c r="O20" s="166">
+      <c r="O20" s="165">
         <v>295000</v>
       </c>
       <c r="Q20" s="138"/>
@@ -6156,7 +6153,7 @@
       <c r="A21" s="128">
         <v>20</v>
       </c>
-      <c r="B21" s="162" t="s">
+      <c r="B21" s="161" t="s">
         <v>148</v>
       </c>
       <c r="C21" s="8" t="s">
@@ -6165,7 +6162,7 @@
       <c r="D21" s="8">
         <v>52.140999999999998</v>
       </c>
-      <c r="E21" s="169" t="s">
+      <c r="E21" s="168" t="s">
         <v>144</v>
       </c>
       <c r="F21" s="129">
@@ -6181,11 +6178,11 @@
       <c r="J21" s="113">
         <v>45984</v>
       </c>
-      <c r="K21" s="165">
+      <c r="K21" s="164">
         <f t="shared" si="1"/>
         <v>45985</v>
       </c>
-      <c r="L21" s="165">
+      <c r="L21" s="164">
         <v>45991</v>
       </c>
       <c r="M21" s="131">
@@ -6196,7 +6193,7 @@
         <f t="shared" si="0"/>
         <v>45993</v>
       </c>
-      <c r="O21" s="166">
+      <c r="O21" s="165">
         <v>594000</v>
       </c>
       <c r="Q21" s="138"/>
@@ -6310,7 +6307,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="B1:P13"/>
+  <dimension ref="B1:P16"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="1.36328125" customWidth="1"/>
@@ -6326,349 +6323,356 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B1" s="203" t="s">
+      <c r="B1" s="202" t="s">
         <v>158</v>
       </c>
-      <c r="C1" s="203"/>
-      <c r="D1" s="203"/>
-      <c r="E1" s="203"/>
-      <c r="F1" s="203"/>
-      <c r="G1" s="203"/>
-      <c r="H1" s="203"/>
-      <c r="I1" s="203"/>
-      <c r="J1" s="203"/>
-      <c r="K1" s="203"/>
-      <c r="L1" s="203"/>
+      <c r="C1" s="202"/>
+      <c r="D1" s="202"/>
+      <c r="E1" s="202"/>
+      <c r="F1" s="202"/>
+      <c r="G1" s="202"/>
+      <c r="H1" s="202"/>
+      <c r="I1" s="202"/>
+      <c r="J1" s="202"/>
+      <c r="K1" s="202"/>
+      <c r="L1" s="202"/>
     </row>
     <row r="2" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B2" s="204" t="s">
+      <c r="B2" s="203" t="s">
         <v>159</v>
       </c>
-      <c r="C2" s="204"/>
-      <c r="D2" s="204"/>
-      <c r="E2" s="204"/>
-      <c r="F2" s="204"/>
-      <c r="G2" s="204"/>
-      <c r="H2" s="204"/>
-      <c r="I2" s="204"/>
-      <c r="J2" s="204"/>
-      <c r="K2" s="204"/>
-      <c r="L2" s="204"/>
+      <c r="C2" s="203"/>
+      <c r="D2" s="203"/>
+      <c r="E2" s="203"/>
+      <c r="F2" s="203"/>
+      <c r="G2" s="203"/>
+      <c r="H2" s="203"/>
+      <c r="I2" s="203"/>
+      <c r="J2" s="203"/>
+      <c r="K2" s="203"/>
+      <c r="L2" s="203"/>
     </row>
     <row r="3" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B3" s="205" t="s">
+      <c r="B3" s="204" t="s">
         <v>114</v>
       </c>
-      <c r="C3" s="205"/>
-      <c r="D3" s="205"/>
-      <c r="E3" s="205"/>
-      <c r="F3" s="205"/>
-      <c r="G3" s="205"/>
-      <c r="H3" s="205"/>
-      <c r="I3" s="205"/>
-      <c r="J3" s="205"/>
-      <c r="K3" s="205"/>
-      <c r="L3" s="205"/>
+      <c r="C3" s="204"/>
+      <c r="D3" s="204"/>
+      <c r="E3" s="204"/>
+      <c r="F3" s="204"/>
+      <c r="G3" s="204"/>
+      <c r="H3" s="204"/>
+      <c r="I3" s="204"/>
+      <c r="J3" s="204"/>
+      <c r="K3" s="204"/>
+      <c r="L3" s="204"/>
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B4" s="206" t="s">
+      <c r="B4" s="205" t="s">
         <v>115</v>
       </c>
-      <c r="C4" s="206"/>
-      <c r="D4" s="206"/>
-      <c r="E4" s="206"/>
-      <c r="F4" s="206"/>
-      <c r="G4" s="206"/>
-      <c r="H4" s="206"/>
-      <c r="I4" s="206"/>
-      <c r="J4" s="206"/>
-      <c r="K4" s="206"/>
-      <c r="L4" s="206"/>
+      <c r="C4" s="205"/>
+      <c r="D4" s="205"/>
+      <c r="E4" s="205"/>
+      <c r="F4" s="205"/>
+      <c r="G4" s="205"/>
+      <c r="H4" s="205"/>
+      <c r="I4" s="205"/>
+      <c r="J4" s="205"/>
+      <c r="K4" s="205"/>
+      <c r="L4" s="205"/>
     </row>
     <row r="5" spans="2:16" ht="16" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B5" s="156" t="s">
+      <c r="B5" s="155" t="s">
         <v>119</v>
       </c>
-      <c r="C5" s="157"/>
-      <c r="D5" s="157"/>
-      <c r="E5" s="157"/>
-      <c r="F5" s="157"/>
-      <c r="G5" s="157"/>
-      <c r="H5" s="157"/>
-      <c r="I5" s="157"/>
-      <c r="J5" s="157"/>
-      <c r="K5" s="158"/>
+      <c r="C5" s="156"/>
+      <c r="D5" s="156"/>
+      <c r="E5" s="156"/>
+      <c r="F5" s="156"/>
+      <c r="G5" s="156"/>
+      <c r="H5" s="156"/>
+      <c r="I5" s="156"/>
+      <c r="J5" s="156"/>
+      <c r="K5" s="157"/>
     </row>
     <row r="6" spans="2:16" ht="43.5" x14ac:dyDescent="0.35">
-      <c r="B6" s="174" t="s">
+      <c r="B6" s="173" t="s">
         <v>162</v>
       </c>
-      <c r="C6" s="174" t="s">
+      <c r="C6" s="173" t="s">
         <v>163</v>
       </c>
-      <c r="D6" s="174" t="s">
+      <c r="D6" s="173" t="s">
         <v>164</v>
       </c>
-      <c r="E6" s="174" t="s">
+      <c r="E6" s="173" t="s">
         <v>165</v>
       </c>
-      <c r="F6" s="174" t="s">
+      <c r="F6" s="173" t="s">
         <v>166</v>
       </c>
-      <c r="G6" s="174" t="s">
+      <c r="G6" s="173" t="s">
         <v>167</v>
       </c>
-      <c r="H6" s="174" t="s">
+      <c r="H6" s="173" t="s">
         <v>116</v>
       </c>
-      <c r="I6" s="174" t="s">
+      <c r="I6" s="173" t="s">
         <v>117</v>
       </c>
-      <c r="J6" s="174" t="s">
+      <c r="J6" s="173" t="s">
         <v>118</v>
       </c>
-      <c r="K6" s="174" t="s">
+      <c r="K6" s="173" t="s">
         <v>168</v>
       </c>
-      <c r="L6" s="174" t="s">
+      <c r="L6" s="173" t="s">
         <v>169</v>
       </c>
-      <c r="M6" s="174" t="s">
+      <c r="M6" s="173" t="s">
         <v>108</v>
       </c>
-      <c r="N6" s="174" t="s">
+      <c r="N6" s="173" t="s">
         <v>170</v>
       </c>
-      <c r="O6" s="174" t="s">
+      <c r="O6" s="173" t="s">
         <v>105</v>
       </c>
-      <c r="P6" s="174" t="s">
+      <c r="P6" s="173" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="7" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B7" s="175">
+      <c r="B7" s="174">
         <v>1</v>
       </c>
-      <c r="C7" s="175" t="s">
+      <c r="C7" s="174" t="s">
         <v>171</v>
       </c>
-      <c r="D7" s="175" t="s">
+      <c r="D7" s="174" t="s">
         <v>172</v>
       </c>
-      <c r="E7" s="175">
-        <v>0.48</v>
-      </c>
-      <c r="F7" s="175" t="s">
+      <c r="E7">
+        <v>480</v>
+      </c>
+      <c r="F7" s="174" t="s">
         <v>173</v>
       </c>
-      <c r="G7" s="175">
-        <v>0</v>
-      </c>
-      <c r="H7" s="176">
+      <c r="G7" s="174">
+        <v>0</v>
+      </c>
+      <c r="H7" s="175">
         <v>45960</v>
       </c>
-      <c r="I7" s="176">
+      <c r="I7" s="175">
         <v>45962</v>
       </c>
-      <c r="J7" s="176">
+      <c r="J7" s="175">
         <v>45964</v>
       </c>
-      <c r="K7" s="176">
+      <c r="K7" s="175">
         <v>45966</v>
       </c>
       <c r="L7" s="8" t="s">
         <v>181</v>
       </c>
-      <c r="M7" s="175" t="s">
+      <c r="M7" s="174" t="s">
         <v>160</v>
       </c>
-      <c r="N7" s="175"/>
-      <c r="O7" s="175" t="s">
+      <c r="N7" s="174"/>
+      <c r="O7" s="174" t="s">
         <v>178</v>
       </c>
-      <c r="P7" s="175" t="s">
+      <c r="P7" s="174" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="8" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B8" s="175">
+      <c r="B8" s="174">
         <v>2</v>
       </c>
-      <c r="C8" s="175" t="s">
+      <c r="C8" s="174" t="s">
         <v>174</v>
       </c>
-      <c r="D8" s="175" t="s">
+      <c r="D8" s="174" t="s">
         <v>171</v>
       </c>
-      <c r="E8" s="175">
-        <v>4.4800000000000004</v>
-      </c>
-      <c r="F8" s="175" t="s">
+      <c r="E8">
+        <v>4480</v>
+      </c>
+      <c r="F8" s="174" t="s">
         <v>173</v>
       </c>
-      <c r="G8" s="175">
+      <c r="G8" s="174">
         <v>11</v>
       </c>
-      <c r="H8" s="176">
+      <c r="H8" s="175">
         <v>45977</v>
       </c>
-      <c r="I8" s="176">
+      <c r="I8" s="175">
         <v>45966</v>
       </c>
-      <c r="J8" s="176">
+      <c r="J8" s="175">
         <v>45974</v>
       </c>
-      <c r="K8" s="176">
+      <c r="K8" s="175">
         <v>45976</v>
       </c>
       <c r="L8" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="M8" s="175" t="s">
+      <c r="M8" s="174" t="s">
         <v>160</v>
       </c>
-      <c r="N8" s="175"/>
-      <c r="O8" s="175" t="s">
+      <c r="N8" s="174"/>
+      <c r="O8" s="174" t="s">
         <v>178</v>
       </c>
-      <c r="P8" s="175" t="s">
+      <c r="P8" s="174" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="9" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B9" s="175">
+      <c r="B9" s="174">
         <v>3</v>
       </c>
-      <c r="C9" s="175" t="s">
+      <c r="C9" s="174" t="s">
         <v>175</v>
       </c>
-      <c r="D9" s="175" t="s">
+      <c r="D9" s="174" t="s">
         <v>174</v>
       </c>
-      <c r="E9" s="175">
-        <v>1.98</v>
-      </c>
-      <c r="F9" s="175" t="s">
+      <c r="E9">
+        <v>1980</v>
+      </c>
+      <c r="F9" s="174" t="s">
         <v>173</v>
       </c>
-      <c r="G9" s="175">
+      <c r="G9" s="174">
         <v>4</v>
       </c>
-      <c r="H9" s="176">
+      <c r="H9" s="175">
         <v>45984</v>
       </c>
-      <c r="I9" s="176">
+      <c r="I9" s="175">
         <v>45976</v>
       </c>
-      <c r="J9" s="176">
+      <c r="J9" s="175">
         <v>45982</v>
       </c>
-      <c r="K9" s="176">
+      <c r="K9" s="175">
         <v>45984</v>
       </c>
       <c r="L9" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="M9" s="175" t="s">
+      <c r="M9" s="174" t="s">
         <v>160</v>
       </c>
-      <c r="N9" s="175"/>
-      <c r="O9" s="175" t="s">
+      <c r="N9" s="174"/>
+      <c r="O9" s="174" t="s">
         <v>180</v>
       </c>
-      <c r="P9" s="175" t="s">
+      <c r="P9" s="174" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="10" spans="2:16" ht="29" x14ac:dyDescent="0.35">
-      <c r="B10" s="175">
+      <c r="B10" s="174">
         <v>4</v>
       </c>
-      <c r="C10" s="175" t="s">
+      <c r="C10" s="174" t="s">
         <v>176</v>
       </c>
-      <c r="D10" s="175" t="s">
+      <c r="D10" s="174" t="s">
         <v>177</v>
       </c>
-      <c r="E10" s="175">
-        <v>2.46</v>
-      </c>
-      <c r="F10" s="175" t="s">
+      <c r="E10">
+        <v>2460</v>
+      </c>
+      <c r="F10" s="174" t="s">
         <v>173</v>
       </c>
-      <c r="G10" s="175">
+      <c r="G10" s="174">
         <v>5</v>
       </c>
-      <c r="H10" s="176">
+      <c r="H10" s="175">
         <v>45971</v>
       </c>
-      <c r="I10" s="176">
+      <c r="I10" s="175">
         <v>45984</v>
       </c>
-      <c r="J10" s="176">
+      <c r="J10" s="175">
         <v>45991</v>
       </c>
-      <c r="K10" s="176">
+      <c r="K10" s="175">
         <v>45993</v>
       </c>
       <c r="L10" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="M10" s="175" t="s">
+      <c r="M10" s="174" t="s">
         <v>160</v>
       </c>
-      <c r="N10" s="175"/>
-      <c r="O10" s="175" t="s">
+      <c r="N10" s="174"/>
+      <c r="O10" s="174" t="s">
         <v>180</v>
       </c>
-      <c r="P10" s="175" t="s">
+      <c r="P10" s="174" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="11" spans="2:16" x14ac:dyDescent="0.35">
-      <c r="B11" s="150"/>
+      <c r="B11" s="149"/>
       <c r="C11" s="8"/>
-      <c r="D11" s="170"/>
-      <c r="E11" s="151"/>
+      <c r="D11" s="169"/>
+      <c r="E11" s="150"/>
       <c r="F11" s="8"/>
       <c r="G11" s="127"/>
-      <c r="H11" s="165"/>
+      <c r="H11" s="164"/>
       <c r="I11" s="127"/>
       <c r="J11" s="127"/>
-      <c r="K11" s="173"/>
-      <c r="L11" s="175"/>
-      <c r="N11" s="175"/>
-      <c r="O11" s="175"/>
-      <c r="P11" s="175"/>
+      <c r="K11" s="172"/>
+      <c r="L11" s="174"/>
+      <c r="N11" s="174"/>
+      <c r="O11" s="174"/>
+      <c r="P11" s="174"/>
     </row>
     <row r="12" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="B12" s="152"/>
-      <c r="C12" s="153"/>
-      <c r="D12" s="171"/>
-      <c r="E12" s="154"/>
-      <c r="F12" s="92"/>
+      <c r="B12" s="151"/>
+      <c r="C12" s="152"/>
+      <c r="D12" s="170"/>
+      <c r="F12" s="153"/>
       <c r="G12" s="92"/>
       <c r="H12" s="92"/>
       <c r="I12" s="92"/>
       <c r="J12" s="92"/>
-      <c r="K12" s="155"/>
-      <c r="L12" s="175"/>
-      <c r="N12" s="175"/>
-      <c r="O12" s="175"/>
-      <c r="P12" s="175"/>
+      <c r="K12" s="154"/>
+      <c r="L12" s="174"/>
+      <c r="N12" s="174"/>
+      <c r="O12" s="174"/>
+      <c r="P12" s="174"/>
     </row>
     <row r="13" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="B13" s="146"/>
       <c r="C13" s="147"/>
-      <c r="D13" s="172"/>
-      <c r="E13" s="148"/>
-      <c r="F13" s="149"/>
-      <c r="G13" s="149"/>
-      <c r="H13" s="149"/>
-      <c r="I13" s="149"/>
-      <c r="J13" s="149"/>
+      <c r="D13" s="171"/>
+      <c r="F13" s="153"/>
+      <c r="G13" s="148"/>
+      <c r="H13" s="148"/>
+      <c r="I13" s="148"/>
+      <c r="J13" s="148"/>
       <c r="K13" s="145"/>
+    </row>
+    <row r="14" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F14" s="153"/>
+    </row>
+    <row r="15" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="F15" s="153"/>
+    </row>
+    <row r="16" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="E16" s="153"/>
     </row>
   </sheetData>
   <mergeCells count="4">
@@ -6966,60 +6970,60 @@
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:28" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A18" s="195" t="s">
+      <c r="A18" s="179" t="s">
         <v>4</v>
       </c>
-      <c r="B18" s="195" t="s">
+      <c r="B18" s="179" t="s">
         <v>42</v>
       </c>
-      <c r="C18" s="191" t="s">
+      <c r="C18" s="176" t="s">
         <v>47</v>
       </c>
-      <c r="D18" s="191" t="s">
+      <c r="D18" s="176" t="s">
         <v>43</v>
       </c>
-      <c r="E18" s="195" t="s">
+      <c r="E18" s="179" t="s">
         <v>8</v>
       </c>
-      <c r="F18" s="182" t="s">
+      <c r="F18" s="191" t="s">
         <v>18</v>
       </c>
-      <c r="G18" s="182"/>
-      <c r="H18" s="182"/>
-      <c r="I18" s="182"/>
-      <c r="J18" s="182"/>
-      <c r="K18" s="185" t="s">
+      <c r="G18" s="191"/>
+      <c r="H18" s="191"/>
+      <c r="I18" s="191"/>
+      <c r="J18" s="191"/>
+      <c r="K18" s="184" t="s">
         <v>19</v>
       </c>
-      <c r="M18" s="191" t="s">
+      <c r="M18" s="176" t="s">
         <v>36</v>
       </c>
-      <c r="O18" s="186" t="s">
+      <c r="O18" s="185" t="s">
         <v>31</v>
       </c>
-      <c r="P18" s="187"/>
-      <c r="Q18" s="187"/>
-      <c r="R18" s="187"/>
-      <c r="S18" s="187"/>
-      <c r="T18" s="188"/>
-      <c r="V18" s="186" t="s">
+      <c r="P18" s="186"/>
+      <c r="Q18" s="186"/>
+      <c r="R18" s="186"/>
+      <c r="S18" s="186"/>
+      <c r="T18" s="187"/>
+      <c r="V18" s="185" t="s">
         <v>30</v>
       </c>
-      <c r="W18" s="187"/>
-      <c r="X18" s="187"/>
-      <c r="Y18" s="187"/>
-      <c r="Z18" s="187"/>
-      <c r="AA18" s="188"/>
-      <c r="AB18" s="189" t="s">
+      <c r="W18" s="186"/>
+      <c r="X18" s="186"/>
+      <c r="Y18" s="186"/>
+      <c r="Z18" s="186"/>
+      <c r="AA18" s="187"/>
+      <c r="AB18" s="188" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="19" spans="1:28" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A19" s="196"/>
-      <c r="B19" s="196"/>
-      <c r="C19" s="193"/>
-      <c r="D19" s="196"/>
-      <c r="E19" s="196"/>
+      <c r="A19" s="180"/>
+      <c r="B19" s="180"/>
+      <c r="C19" s="177"/>
+      <c r="D19" s="180"/>
+      <c r="E19" s="180"/>
       <c r="F19" s="207" t="s">
         <v>40</v>
       </c>
@@ -7031,52 +7035,52 @@
         <v>45</v>
       </c>
       <c r="J19" s="209"/>
-      <c r="K19" s="185"/>
-      <c r="M19" s="192"/>
-      <c r="O19" s="183" t="s">
+      <c r="K19" s="184"/>
+      <c r="M19" s="190"/>
+      <c r="O19" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="P19" s="183" t="s">
+      <c r="P19" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="Q19" s="183" t="s">
+      <c r="Q19" s="182" t="s">
         <v>26</v>
       </c>
-      <c r="R19" s="183" t="s">
+      <c r="R19" s="182" t="s">
         <v>27</v>
       </c>
-      <c r="S19" s="183" t="s">
+      <c r="S19" s="182" t="s">
         <v>28</v>
       </c>
       <c r="T19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="V19" s="183" t="s">
+      <c r="V19" s="182" t="s">
         <v>24</v>
       </c>
-      <c r="W19" s="183" t="s">
+      <c r="W19" s="182" t="s">
         <v>25</v>
       </c>
-      <c r="X19" s="183" t="s">
+      <c r="X19" s="182" t="s">
         <v>26</v>
       </c>
-      <c r="Y19" s="183" t="s">
+      <c r="Y19" s="182" t="s">
         <v>27</v>
       </c>
-      <c r="Z19" s="183" t="s">
+      <c r="Z19" s="182" t="s">
         <v>28</v>
       </c>
       <c r="AA19" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="AB19" s="190"/>
+      <c r="AB19" s="189"/>
     </row>
     <row r="20" spans="1:28" ht="36.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
-      <c r="A20" s="196"/>
-      <c r="B20" s="196"/>
-      <c r="C20" s="193"/>
-      <c r="D20" s="196"/>
-      <c r="E20" s="196"/>
+      <c r="A20" s="180"/>
+      <c r="B20" s="180"/>
+      <c r="C20" s="177"/>
+      <c r="D20" s="180"/>
+      <c r="E20" s="180"/>
       <c r="F20" s="207"/>
       <c r="G20" s="93" t="s">
         <v>10</v>
@@ -7096,17 +7100,17 @@
       <c r="M20" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="O20" s="184"/>
-      <c r="P20" s="184"/>
-      <c r="Q20" s="184"/>
-      <c r="R20" s="184"/>
-      <c r="S20" s="184"/>
+      <c r="O20" s="183"/>
+      <c r="P20" s="183"/>
+      <c r="Q20" s="183"/>
+      <c r="R20" s="183"/>
+      <c r="S20" s="183"/>
       <c r="T20" s="19"/>
-      <c r="V20" s="184"/>
-      <c r="W20" s="184"/>
-      <c r="X20" s="184"/>
-      <c r="Y20" s="184"/>
-      <c r="Z20" s="184"/>
+      <c r="V20" s="183"/>
+      <c r="W20" s="183"/>
+      <c r="X20" s="183"/>
+      <c r="Y20" s="183"/>
+      <c r="Z20" s="183"/>
       <c r="AA20" s="19" t="s">
         <v>20</v>
       </c>
@@ -7127,7 +7131,7 @@
       <c r="D21" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E21" s="210" t="s">
+      <c r="E21" s="206" t="s">
         <v>98</v>
       </c>
       <c r="F21" s="113">
@@ -7201,7 +7205,7 @@
       <c r="D22" s="8" t="s">
         <v>79</v>
       </c>
-      <c r="E22" s="210"/>
+      <c r="E22" s="206"/>
       <c r="F22" s="113">
         <v>45913</v>
       </c>
@@ -7273,7 +7277,7 @@
       <c r="D23" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E23" s="210"/>
+      <c r="E23" s="206"/>
       <c r="F23" s="113">
         <v>45910</v>
       </c>
@@ -7345,7 +7349,7 @@
       <c r="D24" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E24" s="210"/>
+      <c r="E24" s="206"/>
       <c r="F24" s="113">
         <v>45927</v>
       </c>
@@ -7417,7 +7421,7 @@
       <c r="D25" s="8" t="s">
         <v>86</v>
       </c>
-      <c r="E25" s="210"/>
+      <c r="E25" s="206"/>
       <c r="F25" s="113">
         <v>45915</v>
       </c>
@@ -8112,18 +8116,6 @@
     </row>
   </sheetData>
   <mergeCells count="25">
-    <mergeCell ref="E21:E25"/>
-    <mergeCell ref="W19:W20"/>
-    <mergeCell ref="K18:K19"/>
-    <mergeCell ref="M18:M19"/>
-    <mergeCell ref="O18:T18"/>
-    <mergeCell ref="V18:AA18"/>
-    <mergeCell ref="V19:V20"/>
-    <mergeCell ref="A18:A20"/>
-    <mergeCell ref="B18:B20"/>
-    <mergeCell ref="C18:C20"/>
-    <mergeCell ref="D18:D20"/>
-    <mergeCell ref="E18:E20"/>
     <mergeCell ref="AB18:AB19"/>
     <mergeCell ref="F19:F20"/>
     <mergeCell ref="G19:H19"/>
@@ -8137,6 +8129,18 @@
     <mergeCell ref="Q19:Q20"/>
     <mergeCell ref="R19:R20"/>
     <mergeCell ref="S19:S20"/>
+    <mergeCell ref="A18:A20"/>
+    <mergeCell ref="B18:B20"/>
+    <mergeCell ref="C18:C20"/>
+    <mergeCell ref="D18:D20"/>
+    <mergeCell ref="E18:E20"/>
+    <mergeCell ref="E21:E25"/>
+    <mergeCell ref="W19:W20"/>
+    <mergeCell ref="K18:K19"/>
+    <mergeCell ref="M18:M19"/>
+    <mergeCell ref="O18:T18"/>
+    <mergeCell ref="V18:AA18"/>
+    <mergeCell ref="V19:V20"/>
   </mergeCells>
   <conditionalFormatting sqref="C26:C27">
     <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="4DT6">

</xml_diff>